<commit_message>
Add structured case review fields
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -22,18 +22,18 @@
     <sheet name="bucket_policy" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'dialogue_state_review'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bucket_state_representation'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'bucket_transition'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'bucket_predicate_check'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'bucket_boundary_order'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'bucket_modeling'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'bucket_aggregation'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bucket_data_structure'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'bucket_correctness'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'bucket_implementation'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'bucket_debugging'!$A$2:$V$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'bucket_policy'!$A$2:$V$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'dialogue_state_review'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bucket_state_representation'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'bucket_transition'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'bucket_predicate_check'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'bucket_boundary_order'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'bucket_modeling'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'bucket_aggregation'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bucket_data_structure'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'bucket_correctness'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'bucket_implementation'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'bucket_debugging'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'bucket_policy'!$A$2:$AH$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,14 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
+          <t>6. Structured review columns use fixed English options for aggregation: case_decision is accept / revise / drop / discuss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
         </is>
       </c>
     </row>
@@ -542,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -566,6 +573,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -679,6 +699,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -789,6 +869,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -934,6 +1074,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1075,6 +1227,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1226,6 +1390,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1362,6 +1538,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1511,9 +1699,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1524,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1548,6 +1783,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1661,6 +1909,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -1771,6 +2079,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -1923,6 +2291,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2063,6 +2443,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2193,6 +2585,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2359,9 +2763,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2372,7 +2823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2396,6 +2847,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2509,6 +2973,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -2619,6 +3143,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -2778,6 +3362,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2917,6 +3513,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3083,9 +3691,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3096,7 +3751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3120,6 +3775,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3233,6 +3901,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -3343,6 +4071,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -3487,6 +4275,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3623,6 +4423,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3785,9 +4597,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3798,7 +4657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V52"/>
+  <dimension ref="A1:AH52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3822,6 +4681,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3935,6 +4807,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -4045,6 +4977,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -4157,6 +5149,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4266,6 +5270,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4385,6 +5401,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4496,6 +5524,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4611,6 +5651,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4732,6 +5784,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="inlineStr"/>
+      <c r="AH8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4847,6 +5911,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W9" s="2" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr"/>
+      <c r="AG9" s="2" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4965,6 +6041,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AH10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5077,6 +6165,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr"/>
+      <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="inlineStr"/>
+      <c r="AH11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5205,6 +6305,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr"/>
+      <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AH12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5361,6 +6473,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr"/>
+      <c r="Y13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AH13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5492,6 +6616,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr"/>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
+      <c r="AH14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5622,6 +6758,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr"/>
+      <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr"/>
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AH15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5748,6 +6896,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr"/>
+      <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="inlineStr"/>
+      <c r="AH16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5894,6 +7054,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr"/>
+      <c r="Y17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="inlineStr"/>
+      <c r="AH17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6022,6 +7194,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W18" s="2" t="inlineStr"/>
+      <c r="X18" s="2" t="inlineStr"/>
+      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr"/>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr"/>
+      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AG18" s="2" t="inlineStr"/>
+      <c r="AH18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6153,6 +7337,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W19" s="2" t="inlineStr"/>
+      <c r="X19" s="2" t="inlineStr"/>
+      <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr"/>
+      <c r="AA19" s="2" t="inlineStr"/>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="inlineStr"/>
+      <c r="AG19" s="2" t="inlineStr"/>
+      <c r="AH19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6286,6 +7482,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W20" s="2" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr"/>
+      <c r="Y20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="inlineStr"/>
+      <c r="AH20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6426,6 +7634,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" s="2" t="inlineStr"/>
+      <c r="Y21" s="2" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr"/>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6567,6 +7787,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W22" s="2" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr"/>
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="AA22" s="2" t="inlineStr"/>
+      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr"/>
+      <c r="AH22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6699,6 +7931,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W23" s="2" t="inlineStr"/>
+      <c r="X23" s="2" t="inlineStr"/>
+      <c r="Y23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr"/>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AD23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AF23" s="2" t="inlineStr"/>
+      <c r="AG23" s="2" t="inlineStr"/>
+      <c r="AH23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6874,6 +8118,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W24" s="2" t="inlineStr"/>
+      <c r="X24" s="2" t="inlineStr"/>
+      <c r="Y24" s="2" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr"/>
+      <c r="AB24" s="2" t="inlineStr"/>
+      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="inlineStr"/>
+      <c r="AF24" s="2" t="inlineStr"/>
+      <c r="AG24" s="2" t="inlineStr"/>
+      <c r="AH24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7011,6 +8267,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W25" s="2" t="inlineStr"/>
+      <c r="X25" s="2" t="inlineStr"/>
+      <c r="Y25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr"/>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr"/>
+      <c r="AF25" s="2" t="inlineStr"/>
+      <c r="AG25" s="2" t="inlineStr"/>
+      <c r="AH25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7151,6 +8419,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W26" s="2" t="inlineStr"/>
+      <c r="X26" s="2" t="inlineStr"/>
+      <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr"/>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AD26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr"/>
+      <c r="AF26" s="2" t="inlineStr"/>
+      <c r="AG26" s="2" t="inlineStr"/>
+      <c r="AH26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7289,6 +8569,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W27" s="2" t="inlineStr"/>
+      <c r="X27" s="2" t="inlineStr"/>
+      <c r="Y27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr"/>
+      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AD27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr"/>
+      <c r="AF27" s="2" t="inlineStr"/>
+      <c r="AG27" s="2" t="inlineStr"/>
+      <c r="AH27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7419,6 +8711,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr"/>
+      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr"/>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr"/>
+      <c r="AF28" s="2" t="inlineStr"/>
+      <c r="AG28" s="2" t="inlineStr"/>
+      <c r="AH28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7582,6 +8886,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W29" s="2" t="inlineStr"/>
+      <c r="X29" s="2" t="inlineStr"/>
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AA29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AD29" s="2" t="inlineStr"/>
+      <c r="AE29" s="2" t="inlineStr"/>
+      <c r="AF29" s="2" t="inlineStr"/>
+      <c r="AG29" s="2" t="inlineStr"/>
+      <c r="AH29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7741,6 +9057,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr"/>
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AA30" s="2" t="inlineStr"/>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="inlineStr"/>
+      <c r="AF30" s="2" t="inlineStr"/>
+      <c r="AG30" s="2" t="inlineStr"/>
+      <c r="AH30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7890,6 +9218,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W31" s="2" t="inlineStr"/>
+      <c r="X31" s="2" t="inlineStr"/>
+      <c r="Y31" s="2" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr"/>
+      <c r="AA31" s="2" t="inlineStr"/>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr"/>
+      <c r="AF31" s="2" t="inlineStr"/>
+      <c r="AG31" s="2" t="inlineStr"/>
+      <c r="AH31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8032,6 +9372,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W32" s="2" t="inlineStr"/>
+      <c r="X32" s="2" t="inlineStr"/>
+      <c r="Y32" s="2" t="inlineStr"/>
+      <c r="Z32" s="2" t="inlineStr"/>
+      <c r="AA32" s="2" t="inlineStr"/>
+      <c r="AB32" s="2" t="inlineStr"/>
+      <c r="AC32" s="2" t="inlineStr"/>
+      <c r="AD32" s="2" t="inlineStr"/>
+      <c r="AE32" s="2" t="inlineStr"/>
+      <c r="AF32" s="2" t="inlineStr"/>
+      <c r="AG32" s="2" t="inlineStr"/>
+      <c r="AH32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8164,6 +9516,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W33" s="2" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr"/>
+      <c r="Y33" s="2" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr"/>
+      <c r="AB33" s="2" t="inlineStr"/>
+      <c r="AC33" s="2" t="inlineStr"/>
+      <c r="AD33" s="2" t="inlineStr"/>
+      <c r="AE33" s="2" t="inlineStr"/>
+      <c r="AF33" s="2" t="inlineStr"/>
+      <c r="AG33" s="2" t="inlineStr"/>
+      <c r="AH33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8312,6 +9676,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W34" s="2" t="inlineStr"/>
+      <c r="X34" s="2" t="inlineStr"/>
+      <c r="Y34" s="2" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr"/>
+      <c r="AB34" s="2" t="inlineStr"/>
+      <c r="AC34" s="2" t="inlineStr"/>
+      <c r="AD34" s="2" t="inlineStr"/>
+      <c r="AE34" s="2" t="inlineStr"/>
+      <c r="AF34" s="2" t="inlineStr"/>
+      <c r="AG34" s="2" t="inlineStr"/>
+      <c r="AH34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8454,6 +9830,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr"/>
+      <c r="Y35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="AA35" s="2" t="inlineStr"/>
+      <c r="AB35" s="2" t="inlineStr"/>
+      <c r="AC35" s="2" t="inlineStr"/>
+      <c r="AD35" s="2" t="inlineStr"/>
+      <c r="AE35" s="2" t="inlineStr"/>
+      <c r="AF35" s="2" t="inlineStr"/>
+      <c r="AG35" s="2" t="inlineStr"/>
+      <c r="AH35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8608,6 +9996,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W36" s="2" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr"/>
+      <c r="Y36" s="2" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr"/>
+      <c r="AB36" s="2" t="inlineStr"/>
+      <c r="AC36" s="2" t="inlineStr"/>
+      <c r="AD36" s="2" t="inlineStr"/>
+      <c r="AE36" s="2" t="inlineStr"/>
+      <c r="AF36" s="2" t="inlineStr"/>
+      <c r="AG36" s="2" t="inlineStr"/>
+      <c r="AH36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -8745,6 +10145,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr"/>
+      <c r="Y37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="AA37" s="2" t="inlineStr"/>
+      <c r="AB37" s="2" t="inlineStr"/>
+      <c r="AC37" s="2" t="inlineStr"/>
+      <c r="AD37" s="2" t="inlineStr"/>
+      <c r="AE37" s="2" t="inlineStr"/>
+      <c r="AF37" s="2" t="inlineStr"/>
+      <c r="AG37" s="2" t="inlineStr"/>
+      <c r="AH37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -8888,6 +10300,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr"/>
+      <c r="Y38" s="2" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="2" t="inlineStr"/>
+      <c r="AC38" s="2" t="inlineStr"/>
+      <c r="AD38" s="2" t="inlineStr"/>
+      <c r="AE38" s="2" t="inlineStr"/>
+      <c r="AF38" s="2" t="inlineStr"/>
+      <c r="AG38" s="2" t="inlineStr"/>
+      <c r="AH38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9029,6 +10453,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr"/>
+      <c r="Y39" s="2" t="inlineStr"/>
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr"/>
+      <c r="AB39" s="2" t="inlineStr"/>
+      <c r="AC39" s="2" t="inlineStr"/>
+      <c r="AD39" s="2" t="inlineStr"/>
+      <c r="AE39" s="2" t="inlineStr"/>
+      <c r="AF39" s="2" t="inlineStr"/>
+      <c r="AG39" s="2" t="inlineStr"/>
+      <c r="AH39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9180,6 +10616,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr"/>
+      <c r="Y40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr"/>
+      <c r="AB40" s="2" t="inlineStr"/>
+      <c r="AC40" s="2" t="inlineStr"/>
+      <c r="AD40" s="2" t="inlineStr"/>
+      <c r="AE40" s="2" t="inlineStr"/>
+      <c r="AF40" s="2" t="inlineStr"/>
+      <c r="AG40" s="2" t="inlineStr"/>
+      <c r="AH40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9316,6 +10764,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr"/>
+      <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr"/>
+      <c r="AB41" s="2" t="inlineStr"/>
+      <c r="AC41" s="2" t="inlineStr"/>
+      <c r="AD41" s="2" t="inlineStr"/>
+      <c r="AE41" s="2" t="inlineStr"/>
+      <c r="AF41" s="2" t="inlineStr"/>
+      <c r="AG41" s="2" t="inlineStr"/>
+      <c r="AH41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -9465,6 +10925,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr"/>
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr"/>
+      <c r="AA42" s="2" t="inlineStr"/>
+      <c r="AB42" s="2" t="inlineStr"/>
+      <c r="AC42" s="2" t="inlineStr"/>
+      <c r="AD42" s="2" t="inlineStr"/>
+      <c r="AE42" s="2" t="inlineStr"/>
+      <c r="AF42" s="2" t="inlineStr"/>
+      <c r="AG42" s="2" t="inlineStr"/>
+      <c r="AH42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -9615,6 +11087,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr"/>
+      <c r="Y43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr"/>
+      <c r="AB43" s="2" t="inlineStr"/>
+      <c r="AC43" s="2" t="inlineStr"/>
+      <c r="AD43" s="2" t="inlineStr"/>
+      <c r="AE43" s="2" t="inlineStr"/>
+      <c r="AF43" s="2" t="inlineStr"/>
+      <c r="AG43" s="2" t="inlineStr"/>
+      <c r="AH43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -9755,6 +11239,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr"/>
+      <c r="Y44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr"/>
+      <c r="AB44" s="2" t="inlineStr"/>
+      <c r="AC44" s="2" t="inlineStr"/>
+      <c r="AD44" s="2" t="inlineStr"/>
+      <c r="AE44" s="2" t="inlineStr"/>
+      <c r="AF44" s="2" t="inlineStr"/>
+      <c r="AG44" s="2" t="inlineStr"/>
+      <c r="AH44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -9885,6 +11381,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr"/>
+      <c r="Y45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr"/>
+      <c r="AA45" s="2" t="inlineStr"/>
+      <c r="AB45" s="2" t="inlineStr"/>
+      <c r="AC45" s="2" t="inlineStr"/>
+      <c r="AD45" s="2" t="inlineStr"/>
+      <c r="AE45" s="2" t="inlineStr"/>
+      <c r="AF45" s="2" t="inlineStr"/>
+      <c r="AG45" s="2" t="inlineStr"/>
+      <c r="AH45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10051,6 +11559,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr"/>
+      <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="AA46" s="2" t="inlineStr"/>
+      <c r="AB46" s="2" t="inlineStr"/>
+      <c r="AC46" s="2" t="inlineStr"/>
+      <c r="AD46" s="2" t="inlineStr"/>
+      <c r="AE46" s="2" t="inlineStr"/>
+      <c r="AF46" s="2" t="inlineStr"/>
+      <c r="AG46" s="2" t="inlineStr"/>
+      <c r="AH46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -10208,6 +11728,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr"/>
+      <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr"/>
+      <c r="AB47" s="2" t="inlineStr"/>
+      <c r="AC47" s="2" t="inlineStr"/>
+      <c r="AD47" s="2" t="inlineStr"/>
+      <c r="AE47" s="2" t="inlineStr"/>
+      <c r="AF47" s="2" t="inlineStr"/>
+      <c r="AG47" s="2" t="inlineStr"/>
+      <c r="AH47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -10347,6 +11879,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W48" s="2" t="inlineStr"/>
+      <c r="X48" s="2" t="inlineStr"/>
+      <c r="Y48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="AA48" s="2" t="inlineStr"/>
+      <c r="AB48" s="2" t="inlineStr"/>
+      <c r="AC48" s="2" t="inlineStr"/>
+      <c r="AD48" s="2" t="inlineStr"/>
+      <c r="AE48" s="2" t="inlineStr"/>
+      <c r="AF48" s="2" t="inlineStr"/>
+      <c r="AG48" s="2" t="inlineStr"/>
+      <c r="AH48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -10513,6 +12057,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F4、expected_tutor_move=prerequisite_repair 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W49" s="2" t="inlineStr"/>
+      <c r="X49" s="2" t="inlineStr"/>
+      <c r="Y49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr"/>
+      <c r="AB49" s="2" t="inlineStr"/>
+      <c r="AC49" s="2" t="inlineStr"/>
+      <c r="AD49" s="2" t="inlineStr"/>
+      <c r="AE49" s="2" t="inlineStr"/>
+      <c r="AF49" s="2" t="inlineStr"/>
+      <c r="AG49" s="2" t="inlineStr"/>
+      <c r="AH49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -10655,6 +12211,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W50" s="2" t="inlineStr"/>
+      <c r="X50" s="2" t="inlineStr"/>
+      <c r="Y50" s="2" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr"/>
+      <c r="AA50" s="2" t="inlineStr"/>
+      <c r="AB50" s="2" t="inlineStr"/>
+      <c r="AC50" s="2" t="inlineStr"/>
+      <c r="AD50" s="2" t="inlineStr"/>
+      <c r="AE50" s="2" t="inlineStr"/>
+      <c r="AF50" s="2" t="inlineStr"/>
+      <c r="AG50" s="2" t="inlineStr"/>
+      <c r="AH50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -10791,6 +12359,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W51" s="2" t="inlineStr"/>
+      <c r="X51" s="2" t="inlineStr"/>
+      <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr"/>
+      <c r="AA51" s="2" t="inlineStr"/>
+      <c r="AB51" s="2" t="inlineStr"/>
+      <c r="AC51" s="2" t="inlineStr"/>
+      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AE51" s="2" t="inlineStr"/>
+      <c r="AF51" s="2" t="inlineStr"/>
+      <c r="AG51" s="2" t="inlineStr"/>
+      <c r="AH51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -10953,9 +12533,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=safe_redirect 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W52" s="2" t="inlineStr"/>
+      <c r="X52" s="2" t="inlineStr"/>
+      <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr"/>
+      <c r="AA52" s="2" t="inlineStr"/>
+      <c r="AB52" s="2" t="inlineStr"/>
+      <c r="AC52" s="2" t="inlineStr"/>
+      <c r="AD52" s="2" t="inlineStr"/>
+      <c r="AE52" s="2" t="inlineStr"/>
+      <c r="AF52" s="2" t="inlineStr"/>
+      <c r="AG52" s="2" t="inlineStr"/>
+      <c r="AH52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10966,7 +12593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:AH8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10990,6 +12617,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11103,6 +12743,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -11213,6 +12913,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -11325,6 +13085,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -11434,6 +13206,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -11553,6 +13337,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -11664,6 +13460,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -11779,6 +13587,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -11900,9 +13720,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="inlineStr"/>
+      <c r="AH8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11913,7 +13780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11937,6 +13804,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12050,6 +13930,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -12160,6 +14100,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -12277,6 +14277,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -12395,6 +14407,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -12507,6 +14531,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -12635,6 +14671,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=NA、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -12791,9 +14839,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12804,7 +14899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12828,6 +14923,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12941,6 +15049,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -13051,6 +15219,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -13184,6 +15412,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -13314,6 +15554,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -13440,6 +15692,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -13586,6 +15850,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -13714,9 +15990,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13727,7 +16050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13751,6 +16074,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13864,6 +16200,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -13974,6 +16370,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -14107,6 +16563,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -14240,6 +16708,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -14380,6 +16860,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -14521,6 +17013,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -14653,9 +17157,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14666,7 +17217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14690,6 +17241,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14803,6 +17367,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -14913,6 +17537,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -15090,6 +17774,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -15227,6 +17923,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -15367,6 +18075,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -15505,6 +18225,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -15635,9 +18367,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15648,7 +18427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -15672,6 +18451,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15785,6 +18577,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -15895,6 +18747,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -16060,6 +18972,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -16219,6 +19143,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -16368,6 +19304,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -16510,9 +19458,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16523,7 +19518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -16547,6 +19542,19 @@
     <col width="38" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="46" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16660,6 +19668,66 @@
           <t>Coach Review Notes</t>
         </is>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Source Usability</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Context Coherence</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Student Wording Realism</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Followability Label Validity</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Missing Bridge Validity</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden Content Validity</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Success Criteria Validity</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Leakage Boundary Clarity</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Case Decision</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Issue Type</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Coach Fix Suggestion</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer Confidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -16770,6 +19838,66 @@
       <c r="V2" s="4" t="inlineStr">
         <is>
           <t>review_notes_for_coach</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>source_ok</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>context_coherent</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>student_message_realistic</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>followability_ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>missing_bridge_ok</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>forbidden_content_ok</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>success_criteria_ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>leakage_boundary_ok</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>case_decision</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>issue_type</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>coach_fix_suggestion</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_confidence</t>
         </is>
       </c>
     </row>
@@ -16904,6 +20032,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -17052,6 +20192,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F3、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -17194,6 +20346,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -17348,6 +20512,18 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -17485,9 +20661,56 @@
           <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=micro_step 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:V2"/>
+  <autoFilter ref="A2:AH2"/>
+  <dataValidations count="11">
+    <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,partial,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,not_applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"yes,revise,no,unclear"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"accept,revise,drop,discuss"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
+      <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refine dialogue-state calibration cases
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -2237,19 +2237,19 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>学生：算法方向我基本知道，可是代码里数组开多大、从 0 还是 1 开始、初始值设什么经常出错。 我现在不知道该先看思路还是先看代码，所以越写越乱。 我不确定该看题面的哪个限制，所以后面越写越乱。
-AI：先别急着要完整做法。围绕《[NOIP 2005 普及组] 循环》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《[NOIP 2005 普及组] 循环》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我试着顺了样例，可是到中间那一步就断了。
-AI：先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -2389,19 +2389,19 @@
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>学生：我现在不是不会思路，而是实现时总在边界挂掉。样例过了，但换到极小或极大数据就不放心。 我不确定该看题面的哪个限制，所以后面越写越乱。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。
-AI：先别急着要完整做法。围绕《洛谷的文件夹》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《洛谷的文件夹》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我感觉自己在套模板，不确定这个判断是不是对应题意。
-AI：那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -2525,35 +2525,35 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
           <t>学生：题面编号、循环范围和数组大小总对不上，我不知道该先用哪个最小样例来检查。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
-AI：好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫</t>
+          <t>我有点懵，这题里</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -2703,30 +2703,30 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
           <t>学生：我大概知道要怎么做，但一到第一行、最后一行、空情况这些地方就容易写错。 我现在不知道该先看思路还是先看代码，所以越写越乱。 我不确定该看题面的哪个限制，所以后面越写越乱。
-AI：先别急着要完整做法。围绕《[NOIP 2008 普及组] 立体图》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《[NOIP 2008 普及组] 立体图》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我试着顺了样例，可是到中间那一步就断了。
-AI：先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>一个来源应该是已经处理完前面部分后的结果。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -6440,12 +6440,12 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>一个来源应该是已经处理完前面部分后的结果。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>当前阶段</t>
+          <t>来源</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>应该是看哪一边还是旧状态，避免被这轮更新覆盖。</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -7304,12 +7304,12 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>应该是看哪一边还是旧状态，避免被这轮更新覆盖。</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>当前阶段</t>
+          <t>覆盖</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr"/>
@@ -7424,7 +7424,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>另一种情况也要算吗？</t>
+          <t>我知道要保护旧值，但不知道顺序怎么避免覆盖。</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -7597,12 +7597,12 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>另一种情况也要算吗？</t>
+          <t>我知道要保护旧值，但不知道顺序怎么避免覆盖。</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>另一种</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。</t>
+          <t>我能看出要看更新前后，可是不知道哪一个值会被覆盖。</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -7750,12 +7750,12 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。</t>
+          <t>我能看出要看更新前后，可是不知道哪一个值会被覆盖。</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>不确定</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -7873,7 +7873,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。 还分不清新旧值。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。 还分不清新旧值。</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -8081,12 +8081,12 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>不知道</t>
+          <t>不确定</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。 另一个来源我不敢确定。</t>
+          <t>对象我大概知道，可关系怎么连还没想明白。 对象之间怎么连不确定。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。 另一个来源我不敢确定。</t>
+          <t>对象我大概知道，可关系怎么连还没想明白。 对象之间怎么连不确定。</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
@@ -8361,7 +8361,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>我知道题面里有哪些东西，但不知道该抽成哪种关系。 覆盖关系我说不准。</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -8382,12 +8382,12 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>我知道题面里有哪些东西，但不知道该抽成哪种关系。 覆盖关系我说不准。</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>没想明白</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -8532,12 +8532,12 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>不知道</t>
+          <t>不确定</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>对象是时间段还是选择本身？我感觉关系有点反。 覆盖关系我搞反了。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -8674,7 +8674,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>对象是时间段还是选择本身？我感觉关系有点反。 覆盖关系我搞反了。</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -11033,19 +11033,19 @@
       <c r="M43" s="2" t="inlineStr">
         <is>
           <t>学生：算法方向我基本知道，可是代码里数组开多大、从 0 还是 1 开始、初始值设什么经常出错。 我现在不知道该先看思路还是先看代码，所以越写越乱。 我不确定该看题面的哪个限制，所以后面越写越乱。
-AI：先别急着要完整做法。围绕《[NOIP 2005 普及组] 循环》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《[NOIP 2005 普及组] 循环》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我试着顺了样例，可是到中间那一步就断了。
-AI：先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -11185,19 +11185,19 @@
       <c r="M44" s="2" t="inlineStr">
         <is>
           <t>学生：我现在不是不会思路，而是实现时总在边界挂掉。样例过了，但换到极小或极大数据就不放心。 我不确定该看题面的哪个限制，所以后面越写越乱。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。
-AI：先别急着要完整做法。围绕《洛谷的文件夹》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《洛谷的文件夹》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我感觉自己在套模板，不确定这个判断是不是对应题意。
-AI：那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>那先别扩大范围。继续只看这一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>那先别扩大范围。继续只看这一小步：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -11321,35 +11321,35 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
           <t>学生：题面编号、循环范围和数组大小总对不上，我不知道该先用哪个最小样例来检查。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
-AI：好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫</t>
+          <t>我有点懵，这题里</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -11499,30 +11499,30 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
           <t>学生：我大概知道要怎么做，但一到第一行、最后一行、空情况这些地方就容易写错。 我现在不知道该先看思路还是先看代码，所以越写越乱。 我不确定该看题面的哪个限制，所以后面越写越乱。
-AI：先别急着要完整做法。围绕《[NOIP 2008 普及组] 立体图》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。
+AI：先别急着要完整做法。围绕《[NOIP 2008 普及组] 立体图》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
 学生：我试着顺了样例，可是到中间那一步就断了。
-AI：先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>先不用写完整式子。现在只补这个关系：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先不用写完整式子。现在只补这个关系：你先拿最小样例核对一个边界、初值或变量范围。</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>一个来源应该是已经处理完前面部分后的结果。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -14806,12 +14806,12 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>一个来源应该是已经处理完前面部分后的结果。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>当前阶段</t>
+          <t>来源</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
@@ -16509,7 +16509,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>应该是看哪一边还是旧状态，避免被这轮更新覆盖。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -16530,12 +16530,12 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>是不是先记录到当前阶段为止还能成立的情况？</t>
+          <t>应该是看哪一边还是旧状态，避免被这轮更新覆盖。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>当前阶段</t>
+          <t>覆盖</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
@@ -16650,7 +16650,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -16802,7 +16802,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>另一种情况也要算吗？</t>
+          <t>我知道要保护旧值，但不知道顺序怎么避免覆盖。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -16823,12 +16823,12 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>另一种情况也要算吗？</t>
+          <t>我知道要保护旧值，但不知道顺序怎么避免覆盖。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>另一种</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -16955,7 +16955,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。</t>
+          <t>我能看出要看更新前后，可是不知道哪一个值会被覆盖。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -16976,12 +16976,12 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。</t>
+          <t>我能看出要看更新前后，可是不知道哪一个值会被覆盖。</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>不确定</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -17099,7 +17099,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。 还分不清新旧值。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -17120,7 +17120,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>好像和旧值顺序有关，但从大到小还是从小到大我还没想明白。 还分不清新旧值。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -17716,7 +17716,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -17737,12 +17737,12 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>不知道</t>
+          <t>不确定</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -17865,7 +17865,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。 另一个来源我不敢确定。</t>
+          <t>对象我大概知道，可关系怎么连还没想明白。 对象之间怎么连不确定。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>我能想到一个来源，但另一种情况是不是也要单独算，我不确定。 另一个来源我不敢确定。</t>
+          <t>对象我大概知道，可关系怎么连还没想明白。 对象之间怎么连不确定。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -18017,7 +18017,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>我知道题面里有哪些东西，但不知道该抽成哪种关系。 覆盖关系我说不准。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -18038,12 +18038,12 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>这一步好像能从前面接过来，可是分支怎么拆我还没想明白。 我还不会把分支合起来。</t>
+          <t>我知道题面里有哪些东西，但不知道该抽成哪种关系。 覆盖关系我说不准。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>没想明白</t>
+          <t>不知道</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -18167,7 +18167,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -18188,12 +18188,12 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>大概是看前面能不能推过来，但我不知道要不要把另一种情况也算进去。 我怕漏掉另一种情况。</t>
+          <t>我能列出对象，但它们之间到底是覆盖、相邻还是依赖，我不确定。 关系我还没列清。</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>不知道</t>
+          <t>不确定</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -18309,7 +18309,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>对象是时间段还是选择本身？我感觉关系有点反。 覆盖关系我搞反了。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -18330,7 +18330,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>对象是时间段还是选择本身？我感觉关系有点反。 覆盖关系我搞反了。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Clarify bucket sheet review workflow
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -22,18 +22,18 @@
     <sheet name="bucket_policy" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'dialogue_state_review'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bucket_state_representation'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'bucket_transition'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'bucket_predicate_check'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'bucket_boundary_order'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'bucket_modeling'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'bucket_aggregation'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bucket_data_structure'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'bucket_correctness'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'bucket_implementation'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'bucket_debugging'!$A$2:$AH$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'bucket_policy'!$A$2:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'dialogue_state_review'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'bucket_state_representation'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'bucket_transition'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'bucket_predicate_check'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'bucket_boundary_order'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'bucket_modeling'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'bucket_aggregation'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bucket_data_structure'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'bucket_correctness'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'bucket_implementation'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'bucket_debugging'!$A$2:$AJ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'bucket_policy'!$A$2:$AJ$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -527,14 +527,28 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6. Structured review columns use fixed English options for aggregation: case_decision is accept / revise / drop / discuss.</t>
+          <t>6. Prefer filling the bucket sheets; the main sheet is for global browsing. The summary script will aggregate structured review fields from bucket sheets.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
+          <t>7. Structured review columns use fixed English options for aggregation: case_decision is accept / revise / drop / discuss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9. context_ai_reply / prior_ai_scaffold are only for checking whether the student reply follows the previous scaffold, not for judging that AI reply's quality.</t>
         </is>
       </c>
     </row>
@@ -549,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -586,6 +600,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -759,6 +775,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -929,6 +955,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -1086,6 +1122,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1239,6 +1277,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1402,6 +1442,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1550,6 +1592,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1711,9 +1755,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -1759,7 +1805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH6"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1796,6 +1842,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1969,6 +2017,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -2139,6 +2197,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -2303,6 +2371,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2455,6 +2525,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2597,6 +2669,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2775,9 +2849,11 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -2823,7 +2899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH5"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2860,6 +2936,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3033,6 +3111,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -3203,6 +3291,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -3374,6 +3472,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3525,6 +3625,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3703,9 +3805,11 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -3751,7 +3855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH5"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3788,6 +3892,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3961,6 +4067,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -4131,6 +4247,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -4287,6 +4413,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4435,6 +4563,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4609,9 +4739,11 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -4657,7 +4789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH52"/>
+  <dimension ref="A1:AJ52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4694,6 +4826,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4867,6 +5001,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -5037,6 +5181,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -5161,6 +5315,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5282,6 +5438,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -5413,6 +5571,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5536,6 +5696,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -5663,6 +5825,8 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -5796,6 +5960,8 @@
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5923,6 +6089,8 @@
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr"/>
+      <c r="AI9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -6053,6 +6221,8 @@
       <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr"/>
+      <c r="AI10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -6177,6 +6347,8 @@
       <c r="AF11" s="2" t="inlineStr"/>
       <c r="AG11" s="2" t="inlineStr"/>
       <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6317,6 +6489,8 @@
       <c r="AF12" s="2" t="inlineStr"/>
       <c r="AG12" s="2" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr"/>
+      <c r="AI12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6485,6 +6659,8 @@
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="inlineStr"/>
       <c r="AH13" s="2" t="inlineStr"/>
+      <c r="AI13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -6628,6 +6804,8 @@
       <c r="AF14" s="2" t="inlineStr"/>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr"/>
+      <c r="AI14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6770,6 +6948,8 @@
       <c r="AF15" s="2" t="inlineStr"/>
       <c r="AG15" s="2" t="inlineStr"/>
       <c r="AH15" s="2" t="inlineStr"/>
+      <c r="AI15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6908,6 +7088,8 @@
       <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="inlineStr"/>
       <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AI16" s="2" t="inlineStr"/>
+      <c r="AJ16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7066,6 +7248,8 @@
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="inlineStr"/>
       <c r="AH17" s="2" t="inlineStr"/>
+      <c r="AI17" s="2" t="inlineStr"/>
+      <c r="AJ17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7206,6 +7390,8 @@
       <c r="AF18" s="2" t="inlineStr"/>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="inlineStr"/>
+      <c r="AI18" s="2" t="inlineStr"/>
+      <c r="AJ18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7349,6 +7535,8 @@
       <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="inlineStr"/>
       <c r="AH19" s="2" t="inlineStr"/>
+      <c r="AI19" s="2" t="inlineStr"/>
+      <c r="AJ19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7494,6 +7682,8 @@
       <c r="AF20" s="2" t="inlineStr"/>
       <c r="AG20" s="2" t="inlineStr"/>
       <c r="AH20" s="2" t="inlineStr"/>
+      <c r="AI20" s="2" t="inlineStr"/>
+      <c r="AJ20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7646,6 +7836,8 @@
       <c r="AF21" s="2" t="inlineStr"/>
       <c r="AG21" s="2" t="inlineStr"/>
       <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AI21" s="2" t="inlineStr"/>
+      <c r="AJ21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7799,6 +7991,8 @@
       <c r="AF22" s="2" t="inlineStr"/>
       <c r="AG22" s="2" t="inlineStr"/>
       <c r="AH22" s="2" t="inlineStr"/>
+      <c r="AI22" s="2" t="inlineStr"/>
+      <c r="AJ22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7943,6 +8137,8 @@
       <c r="AF23" s="2" t="inlineStr"/>
       <c r="AG23" s="2" t="inlineStr"/>
       <c r="AH23" s="2" t="inlineStr"/>
+      <c r="AI23" s="2" t="inlineStr"/>
+      <c r="AJ23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8130,6 +8326,8 @@
       <c r="AF24" s="2" t="inlineStr"/>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="inlineStr"/>
+      <c r="AI24" s="2" t="inlineStr"/>
+      <c r="AJ24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8279,6 +8477,8 @@
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="inlineStr"/>
       <c r="AH25" s="2" t="inlineStr"/>
+      <c r="AI25" s="2" t="inlineStr"/>
+      <c r="AJ25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8431,6 +8631,8 @@
       <c r="AF26" s="2" t="inlineStr"/>
       <c r="AG26" s="2" t="inlineStr"/>
       <c r="AH26" s="2" t="inlineStr"/>
+      <c r="AI26" s="2" t="inlineStr"/>
+      <c r="AJ26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8581,6 +8783,8 @@
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="inlineStr"/>
       <c r="AH27" s="2" t="inlineStr"/>
+      <c r="AI27" s="2" t="inlineStr"/>
+      <c r="AJ27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8723,6 +8927,8 @@
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr"/>
       <c r="AH28" s="2" t="inlineStr"/>
+      <c r="AI28" s="2" t="inlineStr"/>
+      <c r="AJ28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8898,6 +9104,8 @@
       <c r="AF29" s="2" t="inlineStr"/>
       <c r="AG29" s="2" t="inlineStr"/>
       <c r="AH29" s="2" t="inlineStr"/>
+      <c r="AI29" s="2" t="inlineStr"/>
+      <c r="AJ29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9069,6 +9277,8 @@
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr"/>
       <c r="AH30" s="2" t="inlineStr"/>
+      <c r="AI30" s="2" t="inlineStr"/>
+      <c r="AJ30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9230,6 +9440,8 @@
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
       <c r="AH31" s="2" t="inlineStr"/>
+      <c r="AI31" s="2" t="inlineStr"/>
+      <c r="AJ31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9384,6 +9596,8 @@
       <c r="AF32" s="2" t="inlineStr"/>
       <c r="AG32" s="2" t="inlineStr"/>
       <c r="AH32" s="2" t="inlineStr"/>
+      <c r="AI32" s="2" t="inlineStr"/>
+      <c r="AJ32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9528,6 +9742,8 @@
       <c r="AF33" s="2" t="inlineStr"/>
       <c r="AG33" s="2" t="inlineStr"/>
       <c r="AH33" s="2" t="inlineStr"/>
+      <c r="AI33" s="2" t="inlineStr"/>
+      <c r="AJ33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9688,6 +9904,8 @@
       <c r="AF34" s="2" t="inlineStr"/>
       <c r="AG34" s="2" t="inlineStr"/>
       <c r="AH34" s="2" t="inlineStr"/>
+      <c r="AI34" s="2" t="inlineStr"/>
+      <c r="AJ34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9842,6 +10060,8 @@
       <c r="AF35" s="2" t="inlineStr"/>
       <c r="AG35" s="2" t="inlineStr"/>
       <c r="AH35" s="2" t="inlineStr"/>
+      <c r="AI35" s="2" t="inlineStr"/>
+      <c r="AJ35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10008,6 +10228,8 @@
       <c r="AF36" s="2" t="inlineStr"/>
       <c r="AG36" s="2" t="inlineStr"/>
       <c r="AH36" s="2" t="inlineStr"/>
+      <c r="AI36" s="2" t="inlineStr"/>
+      <c r="AJ36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10157,6 +10379,8 @@
       <c r="AF37" s="2" t="inlineStr"/>
       <c r="AG37" s="2" t="inlineStr"/>
       <c r="AH37" s="2" t="inlineStr"/>
+      <c r="AI37" s="2" t="inlineStr"/>
+      <c r="AJ37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10312,6 +10536,8 @@
       <c r="AF38" s="2" t="inlineStr"/>
       <c r="AG38" s="2" t="inlineStr"/>
       <c r="AH38" s="2" t="inlineStr"/>
+      <c r="AI38" s="2" t="inlineStr"/>
+      <c r="AJ38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10465,6 +10691,8 @@
       <c r="AF39" s="2" t="inlineStr"/>
       <c r="AG39" s="2" t="inlineStr"/>
       <c r="AH39" s="2" t="inlineStr"/>
+      <c r="AI39" s="2" t="inlineStr"/>
+      <c r="AJ39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10628,6 +10856,8 @@
       <c r="AF40" s="2" t="inlineStr"/>
       <c r="AG40" s="2" t="inlineStr"/>
       <c r="AH40" s="2" t="inlineStr"/>
+      <c r="AI40" s="2" t="inlineStr"/>
+      <c r="AJ40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10776,6 +11006,8 @@
       <c r="AF41" s="2" t="inlineStr"/>
       <c r="AG41" s="2" t="inlineStr"/>
       <c r="AH41" s="2" t="inlineStr"/>
+      <c r="AI41" s="2" t="inlineStr"/>
+      <c r="AJ41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10937,6 +11169,8 @@
       <c r="AF42" s="2" t="inlineStr"/>
       <c r="AG42" s="2" t="inlineStr"/>
       <c r="AH42" s="2" t="inlineStr"/>
+      <c r="AI42" s="2" t="inlineStr"/>
+      <c r="AJ42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11099,6 +11333,8 @@
       <c r="AF43" s="2" t="inlineStr"/>
       <c r="AG43" s="2" t="inlineStr"/>
       <c r="AH43" s="2" t="inlineStr"/>
+      <c r="AI43" s="2" t="inlineStr"/>
+      <c r="AJ43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11251,6 +11487,8 @@
       <c r="AF44" s="2" t="inlineStr"/>
       <c r="AG44" s="2" t="inlineStr"/>
       <c r="AH44" s="2" t="inlineStr"/>
+      <c r="AI44" s="2" t="inlineStr"/>
+      <c r="AJ44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11393,6 +11631,8 @@
       <c r="AF45" s="2" t="inlineStr"/>
       <c r="AG45" s="2" t="inlineStr"/>
       <c r="AH45" s="2" t="inlineStr"/>
+      <c r="AI45" s="2" t="inlineStr"/>
+      <c r="AJ45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11571,6 +11811,8 @@
       <c r="AF46" s="2" t="inlineStr"/>
       <c r="AG46" s="2" t="inlineStr"/>
       <c r="AH46" s="2" t="inlineStr"/>
+      <c r="AI46" s="2" t="inlineStr"/>
+      <c r="AJ46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11740,6 +11982,8 @@
       <c r="AF47" s="2" t="inlineStr"/>
       <c r="AG47" s="2" t="inlineStr"/>
       <c r="AH47" s="2" t="inlineStr"/>
+      <c r="AI47" s="2" t="inlineStr"/>
+      <c r="AJ47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11891,6 +12135,8 @@
       <c r="AF48" s="2" t="inlineStr"/>
       <c r="AG48" s="2" t="inlineStr"/>
       <c r="AH48" s="2" t="inlineStr"/>
+      <c r="AI48" s="2" t="inlineStr"/>
+      <c r="AJ48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12069,6 +12315,8 @@
       <c r="AF49" s="2" t="inlineStr"/>
       <c r="AG49" s="2" t="inlineStr"/>
       <c r="AH49" s="2" t="inlineStr"/>
+      <c r="AI49" s="2" t="inlineStr"/>
+      <c r="AJ49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12223,6 +12471,8 @@
       <c r="AF50" s="2" t="inlineStr"/>
       <c r="AG50" s="2" t="inlineStr"/>
       <c r="AH50" s="2" t="inlineStr"/>
+      <c r="AI50" s="2" t="inlineStr"/>
+      <c r="AJ50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12371,6 +12621,8 @@
       <c r="AF51" s="2" t="inlineStr"/>
       <c r="AG51" s="2" t="inlineStr"/>
       <c r="AH51" s="2" t="inlineStr"/>
+      <c r="AI51" s="2" t="inlineStr"/>
+      <c r="AJ51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12545,9 +12797,11 @@
       <c r="AF52" s="2" t="inlineStr"/>
       <c r="AG52" s="2" t="inlineStr"/>
       <c r="AH52" s="2" t="inlineStr"/>
+      <c r="AI52" s="2" t="inlineStr"/>
+      <c r="AJ52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -12593,7 +12847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH8"/>
+  <dimension ref="A1:AJ8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12630,6 +12884,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12803,6 +13059,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -12973,6 +13239,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -13097,6 +13373,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -13218,6 +13496,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -13349,6 +13629,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -13472,6 +13754,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -13599,6 +13883,8 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -13732,9 +14018,11 @@
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -13780,7 +14068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13817,6 +14105,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13990,6 +14280,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -14160,6 +14460,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -14289,6 +14599,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -14419,6 +14731,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -14543,6 +14857,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -14683,6 +14999,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -14851,9 +15169,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -14899,7 +15219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14936,6 +15256,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15109,6 +15431,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -15279,6 +15611,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -15424,6 +15766,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -15566,6 +15910,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -15704,6 +16050,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -15862,6 +16210,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -16002,9 +16352,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -16050,7 +16402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -16087,6 +16439,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16260,6 +16614,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -16430,6 +16794,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -16575,6 +16949,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -16720,6 +17096,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -16872,6 +17250,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -17025,6 +17405,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -17169,9 +17551,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -17217,7 +17601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -17254,6 +17638,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17427,6 +17813,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -17597,6 +17993,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -17786,6 +18192,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -17935,6 +18343,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -18087,6 +18497,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -18237,6 +18649,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -18379,9 +18793,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -18427,7 +18843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH6"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -18464,6 +18880,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18637,6 +19055,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -18807,6 +19235,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -18984,6 +19422,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -19155,6 +19595,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -19316,6 +19758,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -19470,9 +19914,11 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>
@@ -19518,7 +19964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AJ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -19555,6 +20001,8 @@
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="44" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19728,6 +20176,16 @@
           <t>Reviewer Confidence</t>
         </is>
       </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer ID</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>Review Round</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" s="4" t="inlineStr">
@@ -19898,6 +20356,16 @@
       <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>reviewer_confidence</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>reviewer_id</t>
+        </is>
+      </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>review_round</t>
         </is>
       </c>
     </row>
@@ -20044,6 +20512,8 @@
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
       <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -20204,6 +20674,8 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -20358,6 +20830,8 @@
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -20524,6 +20998,8 @@
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -20673,9 +21149,11 @@
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AH2"/>
+  <autoFilter ref="A2:AJ2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
       <formula1>"yes,partial,no"</formula1>

</xml_diff>

<commit_message>
Document case review reviewer metadata
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -541,14 +541,21 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>8. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
+          <t>8. reviewer_id should be coach_A / coach_B / ai_reviewer_1; review_round should be calibration / round1 / adjudication.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>9. context_ai_reply / prior_ai_scaffold are only for checking whether the student reply follows the previous scaffold, not for judging that AI reply's quality.</t>
+          <t>9. This workbook reviews case/source quality only. It is not an AI-response blind review and should not be used to score condition quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10. context_ai_reply / prior_ai_scaffold are only for checking whether the student reply follows the previous scaffold, not for judging that AI reply's quality.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply calibration review fixes
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -2604,30 +2604,30 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
           <t>学生：题面编号、循环范围和数组大小总对不上，我不知道该先用哪个最小样例来检查。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
+AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿一个字符或空格，核对它应该对应几次按键。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
-AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面范围、数组下标、初始可达状态和变量类型对应起来的实现边界桥。</t>
+          <t>缺少把题面中的字符/空格映射到对应按键次数，并据此逐字符累加的实现桥。</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
@@ -2654,9 +2654,9 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用最小样例核对一个下标、初始值或类型范围。
-回复把注意力放在一个实现边界上。
-回复不直接给完整代码补丁。</t>
+          <t>回复让学生先用一个字符或空格核对对应的按键次数。
+回复把注意力放在字符到次数的局部映射上。
+回复不直接给完整代码补丁或整张字符映射表。</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
@@ -6522,17 +6522,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>clarify</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>一个来源应该是已经处理完前面部分后的结果。</t>
+          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>一个来源应该是已经处理完前面部分后的结果。</t>
+          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -6644,14 +6644,14 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>回复引导学生列出当前一步可由哪些更小子问题产生。
-回复让学生先分析一个选择分支或一个前驱来源。
+          <t>回复先请学生把“已处理完前面部分”具体化成一个前驱来源。
+回复让学生用题面动作或选择说出当前量从哪里来。
 回复不直接写完整递推式。</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
+          <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr"/>
@@ -7482,17 +7482,17 @@
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>学生：这里会不会死循环？
-AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -7508,7 +7508,7 @@
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
+          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
@@ -7520,9 +7520,9 @@
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
-回复用一个很小范围检查边界或顺序含义。
-回复不直接给完整模板或边界更新公式。</t>
+          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
+回复用一个很小容量范围检查循环方向是否会复用本轮新值。
+回复不直接给完整背包模板或循环方向结论。</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
@@ -7625,17 +7625,17 @@
       <c r="M20" s="2" t="inlineStr">
         <is>
           <t>学生：顺序总写反。
-AI：先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
+          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
@@ -7667,9 +7667,9 @@
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
-回复用一个很小范围检查边界或顺序含义。
-回复不直接给完整模板或边界更新公式。</t>
+          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
+回复用一个很小容量范围检查循环方向是否会复用本轮新值。
+回复不直接给完整背包模板或循环方向结论。</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -11566,30 +11566,30 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
           <t>学生：题面编号、循环范围和数组大小总对不上，我不知道该先用哪个最小样例来检查。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿最小样例核对一个边界、初值或变量范围。
+AI：先别急着要完整做法。围绕《手机》，我们只拆当前一小步：你先拿一个字符或空格，核对它应该对应几次按键。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
-AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+AI：好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿最小样例核对一个边界、初值或变量范围。</t>
+          <t>好，我们就停在这个局部。你先回答一个更小的问题：你先拿一个字符或空格，核对它应该对应几次按键。</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？输入范围我也没对上。 如果可以的话，能不能先用这题里的一个字符解释该检查哪个下标或输入边界？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面范围、数组下标、初始可达状态和变量类型对应起来的实现边界桥。</t>
+          <t>缺少把题面中的字符/空格映射到对应按键次数，并据此逐字符累加的实现桥。</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
@@ -11616,9 +11616,9 @@
       </c>
       <c r="U45" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用最小样例核对一个下标、初始值或类型范围。
-回复把注意力放在一个实现边界上。
-回复不直接给完整代码补丁。</t>
+          <t>回复让学生先用一个字符或空格核对对应的按键次数。
+回复把注意力放在字符到次数的局部映射上。
+回复不直接给完整代码补丁或整张字符映射表。</t>
         </is>
       </c>
       <c r="V45" s="2" t="inlineStr">
@@ -15032,17 +15032,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>clarify</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>一个来源应该是已经处理完前面部分后的结果。</t>
+          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -15131,7 +15131,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>一个来源应该是已经处理完前面部分后的结果。</t>
+          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -15154,14 +15154,14 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>回复引导学生列出当前一步可由哪些更小子问题产生。
-回复让学生先分析一个选择分支或一个前驱来源。
+          <t>回复先请学生把“已处理完前面部分”具体化成一个前驱来源。
+回复让学生用题面动作或选择说出当前量从哪里来。
 回复不直接写完整递推式。</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Dialogue-state v3 draft. 请复核 followability=F1、expected_tutor_move=advance 与目标 missing bridge 是否一致。</t>
+          <t>Dialogue-state v3 draft. 请复核 followability=F2、expected_tutor_move=clarify 与目标 missing bridge 是否一致。</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr"/>
@@ -16896,17 +16896,17 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>学生：这里会不会死循环？
-AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -16922,7 +16922,7 @@
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
+          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -16934,9 +16934,9 @@
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
-回复用一个很小范围检查边界或顺序含义。
-回复不直接给完整模板或边界更新公式。</t>
+          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
+回复用一个很小容量范围检查循环方向是否会复用本轮新值。
+回复不直接给完整背包模板或循环方向结论。</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
@@ -17039,17 +17039,17 @@
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>学生：顺序总写反。
-AI：先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+AI：先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
+          <t>先别急着要完整做法。围绕《[NOIP 2006 普及组] 开心的金明》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -17069,7 +17069,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
+          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
@@ -17081,9 +17081,9 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
-回复用一个很小范围检查边界或顺序含义。
-回复不直接给完整模板或边界更新公式。</t>
+          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
+回复用一个很小容量范围检查循环方向是否会复用本轮新值。
+回复不直接给完整背包模板或循环方向结论。</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync calibration review artifacts
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -6600,7 +6600,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -7482,17 +7482,17 @@
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>学生：这里会不会死循环？
-AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -7508,7 +7508,7 @@
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
+          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
@@ -7520,9 +7520,9 @@
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
-回复用一个很小容量范围检查循环方向是否会复用本轮新值。
-回复不直接给完整背包模板或循环方向结论。</t>
+          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
+回复用一个很小范围检查边界或顺序含义。
+回复不直接给完整模板或边界更新公式。</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -15131,7 +15131,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -16896,17 +16896,17 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>学生：这里会不会死循环？
-AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+AI：先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断一次更新时，旧值会不会被本轮刚算出的新值覆盖或复用。</t>
+          <t>先别急着要完整做法。围绕《[SCOI2009] 粉刷匠》，我们只拆当前一小步：你先判断更新后哪一边还可能包含答案，或者哪个旧值不能被覆盖。</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -16922,7 +16922,7 @@
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>缺少把循环方向、上一轮旧值和本轮新值复用风险对应起来的关系。</t>
+          <t>缺少把循环不变量、已处理范围和更新方向对应起来的关系。</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -16934,9 +16934,9 @@
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说清一次更新时哪些旧值必须来自上一轮或上一状态。
-回复用一个很小容量范围检查循环方向是否会复用本轮新值。
-回复不直接给完整背包模板或循环方向结论。</t>
+          <t>回复让学生先说清更新前后哪一段仍可能包含答案或仍可被复用。
+回复用一个很小范围检查边界或顺序含义。
+回复不直接给完整模板或边界更新公式。</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Refine calibration case revisions
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -2604,7 +2604,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我这里卡在最基础的地方：空格算几下，字母又怎么数？能先拿一个字母带我核一下吗？ 我先想把一个字母和一个空格的按键次数算对，不然循环写了也不知道对不对；先别给整段代码。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -2627,12 +2627,12 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我这里卡在最基础的地方：空格算几下，字母又怎么数？能先拿一个字母带我核一下吗？ 我先想把一个字母和一个空格的按键次数算对，不然循环写了也不知道对不对；先别给整段代码。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里</t>
+          <t>我这里卡在最基础</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -2642,21 +2642,21 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面中的字符/空格映射到对应按键次数，并据此逐字符累加的实现桥。</t>
+          <t>缺少把题面中的单个字符（字母或空格）映射到按键次数，并把输入逐字符累计的实现桥。</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
           <t>no_complete_code_patch
 no_full_solution
-no_direct_current_bridge</t>
+no_full_keypress_mapping_table</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用一个字符或空格核对对应的按键次数。
-回复把注意力放在字符到次数的局部映射上。
-回复不直接给完整代码补丁或整张字符映射表。</t>
+          <t>回复先选一个字符或空格，让学生根据题面数出对应按键次数。
+回复只建立“单字符映射 -&gt; 逐字符累计”的局部关系。
+回复不直接给完整代码、整张字符映射表或整题总做法。</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>followup_after_partial_answer</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
+          <t>我能想到一个来源，但没对应到具体题面动作。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -6621,15 +6621,19 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
+          <t>我能想到一个来源，但没对应到具体题面动作。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>来源</t>
-        </is>
-      </c>
-      <c r="R13" s="2" t="inlineStr"/>
+          <t>我能想到一个来源</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>学生方向接近，但没有说清分支或条件。</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
           <t>缺少根据题目允许的动作、选择或依赖关系反推转移来源。</t>
@@ -6644,7 +6648,7 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>回复先请学生把“已处理完前面部分”具体化成一个前驱来源。
+          <t>回复先请学生把“前面某个状态”具体化成一个前驱来源。
 回复让学生用题面动作或选择说出当前量从哪里来。
 回复不直接写完整递推式。</t>
         </is>
@@ -11566,7 +11570,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我这里卡在最基础的地方：空格算几下，字母又怎么数？能先拿一个字母带我核一下吗？ 我先想把一个字母和一个空格的按键次数算对，不然循环写了也不知道对不对；先别给整段代码。</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -11589,12 +11593,12 @@
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里空格和字母要怎么对应到次数？ 如果可以的话，能不能先用这题里的一个字符或空格解释它该算几次按键？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我这里卡在最基础的地方：空格算几下，字母又怎么数？能先拿一个字母带我核一下吗？ 我先想把一个字母和一个空格的按键次数算对，不然循环写了也不知道对不对；先别给整段代码。</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，这题里</t>
+          <t>我这里卡在最基础</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -11604,21 +11608,21 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面中的字符/空格映射到对应按键次数，并据此逐字符累加的实现桥。</t>
+          <t>缺少把题面中的单个字符（字母或空格）映射到按键次数，并把输入逐字符累计的实现桥。</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
           <t>no_complete_code_patch
 no_full_solution
-no_direct_current_bridge</t>
+no_full_keypress_mapping_table</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用一个字符或空格核对对应的按键次数。
-回复把注意力放在字符到次数的局部映射上。
-回复不直接给完整代码补丁或整张字符映射表。</t>
+          <t>回复先选一个字符或空格，让学生根据题面数出对应按键次数。
+回复只建立“单字符映射 -&gt; 逐字符累计”的局部关系。
+回复不直接给完整代码、整张字符映射表或整题总做法。</t>
         </is>
       </c>
       <c r="V45" s="2" t="inlineStr">
@@ -15027,7 +15031,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>followup_after_partial_answer</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -15110,7 +15114,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
+          <t>我能想到一个来源，但没对应到具体题面动作。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -15131,15 +15135,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
+          <t>我能想到一个来源，但没对应到具体题面动作。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>来源</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="inlineStr"/>
+          <t>我能想到一个来源</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>学生方向接近，但没有说清分支或条件。</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>缺少根据题目允许的动作、选择或依赖关系反推转移来源。</t>
@@ -15154,7 +15162,7 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>回复先请学生把“已处理完前面部分”具体化成一个前驱来源。
+          <t>回复先请学生把“前面某个状态”具体化成一个前驱来源。
 回复让学生用题面动作或选择说出当前量从哪里来。
 回复不直接写完整递推式。</t>
         </is>

</xml_diff>

<commit_message>
Add dialogue-state review generation pack
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.en.xlsx
@@ -1013,57 +1013,47 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P10709</t>
+          <t>https://www.luogu.com.cn/problem/P1223</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>luogu_p10709_correctness_invariant</t>
+          <t>luogu_p1223_correctness_invariant</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOISG 2024 Prelim] Party
-来源：洛谷 P10709
-题意摘录：James 有 $n$ 个朋友，他想选择其中的 $0$ 个或者更多朋友来参加他的聚会。第 $i$ 个朋友如果参加了他的聚会，会产生 $a_i$ 点快乐值。注意：有些朋友并不想参加聚会，所以他们的 $a_i$ 会是负的。
-然而，他家只有一排 $n$ 个座位，而且因为社交距离，两个人不能坐在相邻的座位上。现在 James 想知道，如果他按照最优方案邀请朋友，这些朋友的快乐值的和最大为多少。
-输入格式摘录：第一行，一个整数 $n$。
-第二行 $n$ 个整数，表示 $a$。
-输出格式摘录：一行一个整数，表示答案。
-样例输入：5
-3 2 -1 4 5
-样例输出：12
-数据范围/提示摘录：### 【样例 #1 解释】
-James 可以邀请第 $1,4,5$ 位朋友。
-### 【样例 #2 解释】
-James 可以邀请唯一一位朋友。
-### 【样例 #3 解释】
-James 可以邀请第 $3,4,6$ 位朋友。
-### 【数据范围】
-|$\text{Subtask}$|分值|特殊性质|
-|:-:|:-:|:-:|
-|$0$|$0$|样例|
-|$1$|$49$|$n\le 3$|
-|$2$|$38$|$n\le 1000$|
-|$3$|$13$|无|
-对于 $100\%$ 的数据，$1 \le n \le 2 \times 10^5,-10^9 \le a_i \le 10^9$。</t>
+          <t>题目：排队接水
+来源：洛谷 P1223
+题意摘录：有 $n$ 个人在一个水龙头前排队接水，假如每个人接水的时间为 $T_i$，请编程找出这 $n$ 个人排队的一种顺序，使得 $n$ 个人的平均等待时间最小。
+一个人的等待时间不包括他的接水时间。
+如果两个人接水的时间相同，编号更小的人应当排在前面。
+输入格式摘录：第一行为一个整数 $n$。
+第二行 $n$ 个整数，第 $i$ 个整数 $T_i$ 表示第 $i$ 个人的接水时间 $T_i$。
+输出格式摘录：输出文件有两行，第一行为一种平均时间最短的排队顺序；第二行为这种排列方案下的平均等待时间（输出结果精确到小数点后两位）。
+样例输入：10 
+56 12 1 99 1000 234 33 55 99 812
+样例输出：3 2 7 8 1 4 9 6 10 5
+291.90
+数据范围/提示摘录：$1\le n \leq 1000$，$1\le t_i \leq 10^6$，不保证 $t_i$ 不重复。</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P10709《[NOISG 2024 Prelim] Party》：James 有 $n$ 个朋友，他想选择其中的 $0$ 个或者更多朋友来参加他的聚会。第 $i$ 个朋友如果参加了他的聚会，会产生 $a_i$ 点快乐值。注意：有些朋友并不想参加聚会，所以他们的 $a_i$ 会是负的。
-然而，他家只有一排 $n$ 个座位，而且因为社交距离，两个人不能坐在相邻的座位上。...</t>
+          <t>洛谷 P1223《排队接水》：有 $n$ 个人在一个水龙头前排队接水，假如每个人接水的时间为 $T_i$，请编程找出这 $n$ 个人排队的一种顺序，使得 $n$ 个人的平均等待时间最小。
+一个人的等待时间不包括他的接水时间。
+如果两个人接水的时间相同，编号更小的人应当排在前面。</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我试着比较两个相邻选择，但不知道要看总目标值还是局部贡献，感觉还没形成交换理由。样例能跟，可是一换顺序我就不知道为什么不会变差，也不知道该先固定哪个局部对象来比较。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>学生：我觉得可以按某种规则先选一个局部最优，但不知道如果换一种选择顺序，会不会影响最终答案。 我不确定该看题面的哪个限制，所以后面越写越乱。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。
-AI：先别急着要完整做法。围绕《[NOISG 2024 Prelim] Part》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
+          <t>学生：我知道可能要让时间短的人先接水，但不会证明。交换两个人顺序时，到底该比较谁的等待时间变化？
+AI：先别急着要完整做法。围绕《排队接水》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
 学生：我感觉自己在套模板，不确定这个判断是不是对应题意。
 AI：那先别扩大范围。继续只看这一小步：你先比较两个相邻选择互换以后，目标值会不会变差。</t>
         </is>
@@ -1080,36 +1070,36 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我试着比较两个相邻选择，但不知道要看总目标值还是局部贡献，感觉还没形成交换理由。样例能跟，可是一换顺序我就不知道为什么不会变差，也不知道该先固定哪个局部对象来比较。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>交换理由</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>缺少把局部选择与全局目标、不变量或交换论证连接起来的正确性桥。</t>
+          <t>缺少把两个相邻人的顺序交换与总等待时间变化连接起来的正确性桥。</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先比较两个局部选择的后果。
-回复引导学生寻找保持不变的量或可以交换的局部结构。
-回复不直接给完整证明。</t>
+          <t>回复让学生只比较相邻两个人 A、B 交换前后的等待时间贡献。
+回复引导学生找出哪个局部顺序不会让总等待时间变大。
+回复不直接给完整排序规则证明或完整贪心结论。</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
@@ -1170,55 +1160,61 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P10728</t>
+          <t>https://www.luogu.com.cn/problem/P1080</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>luogu_p10728_correctness_invariant</t>
+          <t>luogu_p1080_correctness_invariant</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOISG 2023 Qualification] Swords
-来源：洛谷 P10728
-题意摘录：YH 有 $n$ 把剑，第 $i$ 把剑的攻击力为 $a_i$，防御能力为 $b_i$。
-对于一把剑 $i$，如果存在一个 $j(j \not = i)$，使得 $a_i\le a_j$ 且 $b_i\le b_j$，那么 YH 就认为这把剑是无用的。反之，他就认为这把剑是有用的。
-在本题中，我们保证，不可能找到两把剑 $i,j$，使得 $a_i=a_j$ 且 $b_i=b_j$。
-请你帮助 YH 求出这 $n$ 把剑中，有用的剑的数量。
-输入格式摘录：第一行，一个整数 $n$。
-接下来 $n$ 行，每行两个整数 $a_i,b_i$，表示第 $i$ 把剑形的攻击力和防御能力。
-输出格式摘录：一个整数，表示有用的剑**的数量**。
-样例输入：3
-2 3
-1 3
-5 3
-样例输出：1
-数据范围/提示摘录：|$\text{Subtask}$|分值|特殊性质|
-|:-:|:-:|:-:|
-|$1$|$11$|$n\le500$|
-|$2$|$21$|$a_i,b_i\le500$|
-|$3$|$34$|$a_i=i$|
-|$4$|$25$|对于每一个 $1\le i&lt;j\le n$，有 $a_i\not =a_j$|
-|$5$|$9$|无|
-对于所有数据，$1\le n\le100000,1\le a_i,b_i\le10^9$。</t>
+          <t>题目：[NOIP 2012 提高组] 国王游戏
+来源：洛谷 P1080
+题意摘录：恰逢 H 国国庆，国王邀请 $n$ 位大臣来玩一个有奖游戏。首先，他让每个大臣在左、右手上面分别写下一个整数，国王自己也在左、右手上各写一个整数。然后，让这 $n$ 位大臣排成一排，国王站在队伍的最前面。排好队后，所有的大臣都会获得国王奖赏的若干金币，每位大臣获得的金币数分别是：排在该大臣前面的所有人的左手上的数的乘积除以他自己右手上的数，然后向下取整得到的结果。
+国王不希望某一个大臣获得特别多的奖赏，所以他想请你帮他重新安排一下队伍的顺序，使得获得奖赏最多的大臣，所获奖赏尽可能的少。注意，国王的位置始终在队伍的最前面。
+输入格式摘录：第一行包含一个整数 $n$，表示大臣的人数。
+第二行包含两个整数 $a$ 和 $b$，之间用一个空格隔开，分别表示国王左手和右手上的整数。
+接下来 $n$ 行，每行包含两个整数 $a$ 和 $b$，之间用一个空格隔开，分别表示每个大臣左手和右手上的整数。
+输出格式摘录：一个整数，表示重新排列后的队伍中获奖赏最多的大臣所获得的金币数。
+样例输入：3 
+1 1 
+2 3 
+7 4 
+4 6
+样例输出：2
+数据范围/提示摘录：**【输入输出样例说明】**
+按 $1$、$2$、$3$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $1$、$3$、$2$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $2$、$1$、$3$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $2$、$3$、$1$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $9$；
+按 $3$、$1$、$2$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；  
+按 $3$、$2$、$1$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $9$。
+因此，奖赏最多的大臣最少获得 $2$ 个金币，答案输出 $2$。
+**【数据范围】**
+对于 $20\%$ 的数据，有 $1 \le n \le 10,0 &lt; a,b &lt; 8$；
+对于 $40\%$ 的数据，有 $1 \le n \le 20,0 &lt; a,b &lt; 8$；
+对于 $60\%$ 的数据，有 $1 \le n \le 100$；
+对于 $60\%$ 的数据，保证答案不超过 $10^9$；
+对于 $100\%$...</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P10728《[NOISG 2023 Qualification] Swords》：YH 有 $n$ 把剑，第 $i$ 把剑的攻击力为 $a_i$，防御能力为 $b_i$。
-对于一把剑 $i$，如果存在一个 $j(j \not = i)$，使得 $a_i\le a_j$ 且 $b_i\le b_j$，那么 YH 就认为这把剑是无用的。反之，他就认为这把剑是有用的。...</t>
+          <t>洛谷 P1080《[NOIP 2012 提高组] 国王游戏》：恰逢 H 国国庆，国王邀请 $n$ 位大臣来玩一个有奖游戏。首先，他让每个大臣在左、右手上面分别写下一个整数，国王自己也在左、右手上各写一个整数。然后，让这 $n$ 位大臣排成一排，国王站在队伍的最前面。排好队后，所有的大臣都会获得国王奖赏的若干金币，每位大臣获得的金币数分别是：排在该大臣前面的所有人的左手上的数的乘积除以他自己右手上的数，然后向下取整得到的结果。
+国王不希望某一个大臣获得特别多的奖赏，所以他想请你帮他重新安排一下队伍的顺序，使得获得奖赏最多的大臣，所获奖赏...</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>如果把这两个选择顺序换一下，我不确定哪个量不会变差。样例能跟，但证明这一步不会写，我想先确认比较的对象到底是哪一个，再判断全局目标有没有受影响。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>学生：我能写出一个看起来合理的策略，但说不清它保持了什么不变量，所以不敢相信。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《[NOISG 2023 Qualificatio》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
+          <t>学生：国王游戏里我能想到要排序，但不知道为什么这样排。只交换相邻两个大臣时，应该比较哪几个奖励值？
+AI：先别急着要完整做法。围绕《[NOIP 2012 提高组] 国王游戏》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
 AI：好，我们就停在这个局部。你先回答一个更小的问题：你先比较两个相邻选择互换以后，目标值会不会变差。</t>
         </is>
@@ -1235,36 +1231,36 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>如果把这两个选择顺序换一下，我不确定哪个量不会变差。样例能跟，但证明这一步不会写，我想先确认比较的对象到底是哪一个，再判断全局目标有没有受影响。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不会变差</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>缺少把局部选择与全局目标、不变量或交换论证连接起来的正确性桥。</t>
+          <t>缺少把相邻两个大臣交换前后的局部最坏奖励与全局最大值控制连接起来的正确性桥。</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先比较两个局部选择的后果。
-回复引导学生寻找保持不变的量或可以交换的局部结构。
-回复不直接给完整证明。</t>
+          <t>回复让学生固定其他人，只比较相邻两个大臣交换前后的局部最坏奖励。
+回复引导学生观察交换只影响这两个位置相关的奖励项。
+回复不直接给完整排序关键字或完整交换证明。</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -1377,7 +1373,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 我对《[CSP-J 2024] 小木棍》的整体思路大概能跟，但代码里这个更新顺序一变结果就不一样。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我能猜到要保持某个不变量，但不知道相邻两步交换后到底保持了什么，为什么答案不会更差。现在我只是凭直觉说贪心可行，换一个样例就说不清理由，也不知道该比较哪两个局部方案。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -1400,17 +1396,17 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 我对《[CSP-J 2024] 小木棍》的整体思路大概能跟，但代码里这个更新顺序一变结果就不一样。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我能猜到要保持某个不变量，但不知道相邻两步交换后到底保持了什么，为什么答案不会更差。现在我只是凭直觉说贪心可行，换一个样例就说不清理由，也不知道该比较哪两个局部方案。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不变量</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -1420,9 +1416,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -1527,7 +1523,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我现在只会说这个贪心看起来对，但说不出局部选择换一下会不会影响全局目标。能不能先让我比较一个很小的相邻交换，看交换前后哪个量没有变差，再决定证明方向？</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1550,17 +1546,17 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我现在只会说这个贪心看起来对，但说不出局部选择换一下会不会影响全局目标。能不能先让我比较一个很小的相邻交换，看交换前后哪个量没有变差，再决定证明方向？</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>全局目标</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1570,9 +1566,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -1690,7 +1686,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我想用交换法想这题，但卡在比较两种相邻选择：到底要证明哪个指标不变或不变差？我怕一上来就写证明会变成背模板，所以想先看一个局部比较，再慢慢推广到整体。</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1713,17 +1709,17 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我想用交换法想这题，但卡在比较两种相邻选择：到底要证明哪个指标不变或不变差？我怕一上来就写证明会变成背模板，所以想先看一个局部比较，再慢慢推广到整体。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不变差</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -1733,9 +1729,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -2349,9 +2345,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -2503,9 +2499,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -2647,9 +2643,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_full_keypress_mapping_table</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not provide the full keypress mapping table</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -2784,7 +2780,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>立体图里一个方块画到字符图上时，我不知道单个字符位置到底对应题面里的哪一格、哪条边或哪个角。样例图我能看，但自己画时坐标就乱了，尤其不知道先核对哪个局部字符。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -2807,36 +2803,36 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>立体图里一个方块画到字符图上时，我不知道单个字符位置到底对应题面里的哪一格、哪条边或哪个角。样例图我能看，但自己画时坐标就乱了，尤其不知道先核对哪个局部字符。</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>没懂</t>
+          <t>单个字符位置</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面范围、数组下标、初始可达状态和变量类型对应起来的实现边界桥。</t>
+          <t>缺少把输出图中单个字符位置、题面方块的格子/边/角以及循环坐标对应起来的实现边界桥。</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用最小样例核对一个下标、初始值或类型范围。
-回复把注意力放在一个实现边界上。
-回复不直接给完整代码补丁。</t>
+          <t>回复先选一个最小方块或一个字符位置，让学生判断它对应题面中的哪一格、哪条边或哪个角。
+回复把注意力放在输出坐标、字符位置和题面对象的局部映射上。
+回复不直接给完整画图代码或完整字符模板。</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -3407,7 +3403,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>你说的维护量/不变量我没太理解，能不能先说它在题面里对应什么？ 我可能不是这一步不会写，而是前面那个概念就没有搭起来。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我知道要调试，但不知道“最小反例”该怎么选。能不能先让我挑一个很小输入，看哪个中间量应该是多少？我现在不是想改完整代码，只想把错误缩小到一步。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -3430,17 +3426,17 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>你说的维护量/不变量我没太理解，能不能先说它在题面里对应什么？ 我可能不是这一步不会写，而是前面那个概念就没有搭起来。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我知道要调试，但不知道“最小反例”该怎么选。能不能先让我挑一个很小输入，看哪个中间量应该是多少？我现在不是想改完整代码，只想把错误缩小到一步。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>没太理解</t>
+          <t>最小反例</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -3450,9 +3446,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -3560,7 +3556,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。 我现在愿意自己继续推，但需要一个不会直接暴露答案的提示。最好是让我对着一个最小样例说出下一步，而不是直接告诉我完整模板。</t>
+          <t>这题我样例能跟一点，但不知道该先手算哪一秒、哪个魔法值或距离变量。能先帮我把检查点缩小吗？我现在调试时只会整段跑，看到 WA 也不知道是闪烁、休息还是跑步那一步错了。最好先让我对一个很小时间点写出一个中间值，而不是直接告诉我完整做法。比如只看前两三秒，我也不确定该记录“当前最远距离”还是“剩余魔法”。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -3583,17 +3579,17 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。 我现在愿意自己继续推，但需要一个不会直接暴露答案的提示。最好是让我对着一个最小样例说出下一步，而不是直接告诉我完整模板。</t>
+          <t>这题我样例能跟一点，但不知道该先手算哪一秒、哪个魔法值或距离变量。能先帮我把检查点缩小吗？我现在调试时只会整段跑，看到 WA 也不知道是闪烁、休息还是跑步那一步错了。最好先让我对一个很小时间点写出一个中间值，而不是直接告诉我完整做法。比如只看前两三秒，我也不确定该记录“当前最远距离”还是“剩余魔法”。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫</t>
+          <t>检查点</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -3603,9 +3599,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -3740,7 +3736,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[CSP-J 2021] 网络连接》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。 我已经试过按题面手算一个小例子，但算到中间就不知道该记录哪个量，代码里也不知道该检查哪一行。你先别直接给完整公式，帮我把这个小关系拆清楚就行。</t>
+          <t>网络连接这题我不知道该造哪种最小坏地址来查错，也不知道该先检查解析结果还是连接表。比如样例能过，但一遇到前导零、端口范围或重复 Server，我就不知道该打印哪一步。你先别直接改代码，帮我把一个最小坏样例和要看的中间结果定下来。最好只选一种错误类型，让我判断它应该先输出 ERR、FAIL 还是某个编号。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -3763,17 +3759,17 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[CSP-J 2021] 网络连接》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。 我已经试过按题面手算一个小例子，但算到中间就不知道该记录哪个量，代码里也不知道该检查哪一行。你先别直接给完整公式，帮我把这个小关系拆清楚就行。</t>
+          <t>网络连接这题我不知道该造哪种最小坏地址来查错，也不知道该先检查解析结果还是连接表。比如样例能过，但一遇到前导零、端口范围或重复 Server，我就不知道该打印哪一步。你先别直接改代码，帮我把一个最小坏样例和要看的中间结果定下来。最好只选一种错误类型，让我判断它应该先输出 ERR、FAIL 还是某个编号。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>没懂</t>
+          <t>最小坏地址</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -3783,9 +3779,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -4391,9 +4387,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -4541,9 +4537,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -4717,9 +4713,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -5293,9 +5289,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -5416,9 +5412,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -5549,9 +5545,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -5674,9 +5670,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -5803,9 +5799,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -5938,9 +5934,9 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
@@ -6067,9 +6063,9 @@
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
@@ -6199,9 +6195,9 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -6325,9 +6321,9 @@
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -6467,9 +6463,9 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -6641,9 +6637,9 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
@@ -6786,9 +6782,9 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -6930,9 +6926,9 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
@@ -7070,9 +7066,9 @@
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
@@ -7230,9 +7226,9 @@
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
@@ -7372,9 +7368,9 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -7517,9 +7513,9 @@
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
@@ -7664,9 +7660,9 @@
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
@@ -7818,9 +7814,9 @@
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -7973,9 +7969,9 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
@@ -8119,9 +8115,9 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
@@ -8308,9 +8304,9 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
@@ -8459,9 +8455,9 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
@@ -8613,9 +8609,9 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -8765,9 +8761,9 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -8909,9 +8905,9 @@
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U28" s="2" t="inlineStr">
@@ -9045,7 +9041,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>对 [L,R] 加 X 的影响我能看出来，但不知道标记应该落在 L、R 还是抵消位置。这里我经常写成凭感觉加减。</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -9066,17 +9062,17 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>对 [L,R] 加 X 的影响我能看出来，但不知道标记应该落在 L、R 还是抵消位置。这里我经常写成凭感觉加减。</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>另一边</t>
+          <t>抵消位置</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -9086,9 +9082,9 @@
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr">
@@ -9218,7 +9214,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我能看出一次操作会影响一路上的值，但不知道哪些位置是直接加，哪些位置是为了抵消。这里换一个询问我就乱。</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -9239,17 +9235,17 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我能看出一次操作会影响一路上的值，但不知道哪些位置是直接加，哪些位置是为了抵消。这里换一个询问我就乱。</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>为了抵消</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr">
@@ -9259,9 +9255,9 @@
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr">
@@ -9381,7 +9377,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>单个星球或区间的影响我能跟，但要把很多次影响汇总起来时，我不知道应该在哪些位置打标记。</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -9402,17 +9398,17 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>单个星球或区间的影响我能跟，但要把很多次影响汇总起来时，我不知道应该在哪些位置打标记。</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>打标记</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S31" s="2" t="inlineStr">
@@ -9422,9 +9418,9 @@
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
@@ -9537,7 +9533,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>路径上的贡献怎么累起来我懂一点，但到前缀汇总或公共点附近时，不知道加减点应该放在哪里。</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -9558,17 +9554,17 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>路径上的贡献怎么累起来我懂一点，但到前缀汇总或公共点附近时，不知道加减点应该放在哪里。</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>另一边</t>
+          <t>加减点</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
@@ -9578,9 +9574,9 @@
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
@@ -9683,7 +9679,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我知道要 update/query，但不知道结构里每个节点到底该存什么摘要，才能回答题目要的数量或最值。</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -9704,17 +9700,17 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我知道要 update/query，但不知道结构里每个节点到底该存什么摘要，才能回答题目要的数量或最值。</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>存什么摘要</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S33" s="2" t="inlineStr">
@@ -9724,9 +9720,9 @@
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U33" s="2" t="inlineStr">
@@ -9845,7 +9841,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>一次修改之后，节点里的值要怎么保持正确我没想清。查询时为什么能直接拿这些维护量拼出答案？</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -9866,17 +9862,17 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>一次修改之后，节点里的值要怎么保持正确我没想清。查询时为什么能直接拿这些维护量拼出答案？</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>维护量</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
@@ -9886,9 +9882,9 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
@@ -10001,7 +9997,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道该打印哪个量。</t>
+          <t>我写了个小版本，query 输出和手算差一点。我想先知道一次 update 后，结构里哪个摘要量应该发生变化。</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -10022,17 +10018,17 @@
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道该打印哪个量。</t>
+          <t>我写了个小版本，query 输出和手算差一点。我想先知道一次 update 后，结构里哪个摘要量应该发生变化。</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>中间量</t>
+          <t>摘要量</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
@@ -10042,9 +10038,9 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr">
@@ -10169,7 +10165,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我怀疑不是单纯少写一行。</t>
+          <t>我不太明白查询为什么能由这些维护量拼出来。是不是要先确认每个节点维护的对象和合并含义？</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -10190,17 +10186,17 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我怀疑不是单纯少写一行。</t>
+          <t>我不太明白查询为什么能由这些维护量拼出来。是不是要先确认每个节点维护的对象和合并含义？</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>合并含义</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S36" s="2" t="inlineStr">
@@ -10210,9 +10206,9 @@
       </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U36" s="2" t="inlineStr">
@@ -10280,97 +10276,106 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P2672</t>
+          <t>https://www.luogu.com.cn/problem/P3374</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>luogu_p2672_data_structure_operation_semantics</t>
+          <t>luogu_p3374_data_structure_operation_semantics</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOIP 2015 普及组] 推销员
-来源：洛谷 P2672
-题意摘录：阿明是一名推销员，他奉命到螺丝街推销他们公司的产品。螺丝街是一条死胡同，出口与入口是同一个，街道的一侧是围墙，另一侧是住户。螺丝街一共有 $N$ 家住户，第 $i$ 家住户到入口的距离为 $S_i$ 米。由于同一栋房子里可以有多家住户，所以可能有多家住户与入口的距离相等。阿明会从入口进入，依次向螺丝街的 $X$ 家住户推销产品，然后再原路走出去。
-阿明每走 $1$ 米就会积累 $1$ 点疲劳值，向第 $i$ 家住户推销产品会积累 $A_i$ 点疲劳值。阿明是工作狂，他想知道，对于不同的 $X$，在不走多余的路的前提下，他最多可以积累多少点疲劳值。
-输入格式摘录：第一行有一个正整数 $N$，表示螺丝街住户的数量。
-接下来的一行有 $N$ 个非负整数，其中第 $i$ 个整数 $S_i$ 表示第 $i$ 家住户到入口的距离。数据保证 $S_1 \le S_2 \le \cdots \le S_n &lt;10^8$。
-接下来的一行有 $N$ 个正整数，其中第 $i$ 个整数 $A_i$ 表示向第 $i$ 户住户推销产品会积累的疲劳值。数据保证 $A_i&lt;1000$。
-输出格式摘录：输出 $N$ 行，每行一个正整数，第 $i$ 行整数表示当 $X=i$ 时，阿明最多积累的疲劳值。
-样例输入：5
-1 2 3 4 5
-1 2 3 4 5
-样例输出：15
-19
-22
-24
-25
-数据范围/提示摘录：**输入输出样例 1 说明**
-$X=1$：向住户 $5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值为 $5$，总疲劳值为 $15$。
-$X=2$：向住户 $4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值为 $4+5$，总疲劳值为 $5+5+4+5=19$。
-$X=3$：向住户 $3,4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值 $3+4+5$，总疲劳值为 $5+5+3+4+5=22$。
-$X=4$：向住户 $2,3,4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值 $2+3+4+5$，总疲劳值 $5+5+2+3+4+5=24$。...</t>
+          <t>题目：【模板】树状数组 1
+来源：洛谷 P3374
+题意摘录：如题，已知一个数列，你需要进行下面两种操作：
+- 将某一个数加上 $x$；
+- 求出某区间每一个数的和。
+输入格式摘录：第一行包含两个正整数 $n,m$，分别表示该数列数字的个数和操作的总个数。   
+第二行包含 $n$ 个用空格分隔的整数，其中第 $i$ 个数字表示数列第 $i$ 项的初始值。
+接下来 $m$ 行每行包含 $3$ 个整数，表示一个操作，具体如下：
+- `1 x k`  含义：将第 $x$ 个数加上 $k$；
+- `2 x y`  含义：输出区间 $[x,y]$ 内每个数的和。
+输出格式摘录：输出包含若干行整数，即为所有操作 $2$ 的结果。
+样例输入：5 5
+1 5 4 2 3
+1 1 3
+2 2 5
+1 3 -1
+1 4 2
+2 1 4
+样例输出：14
+16
+数据范围/提示摘录：【数据范围】
+对于 $30\%$ 的数据，$1 \le n \le 8$，$1\le m \le 10$；   
+对于 $70\%$ 的数据，$1\le n,m \le 10^4$；   
+对于 $100\%$ 的数据，$1\le n,m \le 5\times 10^5$，$1\le x\le y\le n$，$-2^{31}\le k&lt;2^{31}$。
+数据保证对于任意时刻，$a$ 的任意子区间（包括长度为 $1$ 和 $n$ 的子区间）和均在 $[-2^{31}, 2^{31})$ 范围内。
+样例说明：
+ ![](https://cdn.luogu.com.cn/upload/pic/2256.png) 
+故输出结果 $14$ 和 $16$。</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P2672《[NOIP 2015 普及组] 推销员》：阿明是一名推销员，他奉命到螺丝街推销他们公司的产品。螺丝街是一条死胡同，出口与入口是同一个，街道的一侧是围墙，另一侧是住户。螺丝街一共有 $N$ 家住户，第 $i$ 家住户到入口的距离为 $S_i$ 米。由于同一栋房子里可以有多家住户，所以可能有多家住户与入口的距离相等。...</t>
+          <t>洛谷 P3374《【模板】树状数组 1》：如题，已知一个数列，你需要进行下面两种操作：
+- 将某一个数加上 $x$；
+- 求出某区间每一个数的和。</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 更新顺序一变结果就不同。</t>
+          <t>更新后结果不稳，我怀疑不是下标问题，而是某个维护量没更新对。应该先检查哪个摘要量？</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>学生：我不清楚一次修改以后，结构里哪些量需要跟着变。 我总觉得差一步。
-AI：先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>学生：我知道有单点加和区间求和，但树状数组里面维护的到底是什么？update 之后 query 为什么还能算区间和？
+AI：先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 更新顺序一变结果就不同。</t>
+          <t>更新后结果不稳，我怀疑不是下标问题，而是某个维护量没更新对。应该先检查哪个摘要量？</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>维护量</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>缺少把数据结构节点、集合或队列中的值与题目需要查询/更新的信息对应起来的关系。</t>
+          <t>缺少把单点修改、前缀和查询以及数据结构内部维护的摘要量对应起来的关系。</t>
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说明一次 update/query 后应保持什么摘要不变量。
-回复用一个极小局部操作检查维护语义。
-回复不直接给完整数据结构操作模板。</t>
+          <t>回复让学生先说明一次 update 后哪些前缀/摘要信息应随之改变。
+回复用一个极小数组检查 query 需要从哪些维护量组合出区间和。
+回复不直接给完整树状数组模板或完整 lowbit 操作序列。</t>
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr">
@@ -10431,57 +10436,47 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P10709</t>
+          <t>https://www.luogu.com.cn/problem/P1223</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>luogu_p10709_correctness_invariant</t>
+          <t>luogu_p1223_correctness_invariant</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOISG 2024 Prelim] Party
-来源：洛谷 P10709
-题意摘录：James 有 $n$ 个朋友，他想选择其中的 $0$ 个或者更多朋友来参加他的聚会。第 $i$ 个朋友如果参加了他的聚会，会产生 $a_i$ 点快乐值。注意：有些朋友并不想参加聚会，所以他们的 $a_i$ 会是负的。
-然而，他家只有一排 $n$ 个座位，而且因为社交距离，两个人不能坐在相邻的座位上。现在 James 想知道，如果他按照最优方案邀请朋友，这些朋友的快乐值的和最大为多少。
-输入格式摘录：第一行，一个整数 $n$。
-第二行 $n$ 个整数，表示 $a$。
-输出格式摘录：一行一个整数，表示答案。
-样例输入：5
-3 2 -1 4 5
-样例输出：12
-数据范围/提示摘录：### 【样例 #1 解释】
-James 可以邀请第 $1,4,5$ 位朋友。
-### 【样例 #2 解释】
-James 可以邀请唯一一位朋友。
-### 【样例 #3 解释】
-James 可以邀请第 $3,4,6$ 位朋友。
-### 【数据范围】
-|$\text{Subtask}$|分值|特殊性质|
-|:-:|:-:|:-:|
-|$0$|$0$|样例|
-|$1$|$49$|$n\le 3$|
-|$2$|$38$|$n\le 1000$|
-|$3$|$13$|无|
-对于 $100\%$ 的数据，$1 \le n \le 2 \times 10^5,-10^9 \le a_i \le 10^9$。</t>
+          <t>题目：排队接水
+来源：洛谷 P1223
+题意摘录：有 $n$ 个人在一个水龙头前排队接水，假如每个人接水的时间为 $T_i$，请编程找出这 $n$ 个人排队的一种顺序，使得 $n$ 个人的平均等待时间最小。
+一个人的等待时间不包括他的接水时间。
+如果两个人接水的时间相同，编号更小的人应当排在前面。
+输入格式摘录：第一行为一个整数 $n$。
+第二行 $n$ 个整数，第 $i$ 个整数 $T_i$ 表示第 $i$ 个人的接水时间 $T_i$。
+输出格式摘录：输出文件有两行，第一行为一种平均时间最短的排队顺序；第二行为这种排列方案下的平均等待时间（输出结果精确到小数点后两位）。
+样例输入：10 
+56 12 1 99 1000 234 33 55 99 812
+样例输出：3 2 7 8 1 4 9 6 10 5
+291.90
+数据范围/提示摘录：$1\le n \leq 1000$，$1\le t_i \leq 10^6$，不保证 $t_i$ 不重复。</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P10709《[NOISG 2024 Prelim] Party》：James 有 $n$ 个朋友，他想选择其中的 $0$ 个或者更多朋友来参加他的聚会。第 $i$ 个朋友如果参加了他的聚会，会产生 $a_i$ 点快乐值。注意：有些朋友并不想参加聚会，所以他们的 $a_i$ 会是负的。
-然而，他家只有一排 $n$ 个座位，而且因为社交距离，两个人不能坐在相邻的座位上。...</t>
+          <t>洛谷 P1223《排队接水》：有 $n$ 个人在一个水龙头前排队接水，假如每个人接水的时间为 $T_i$，请编程找出这 $n$ 个人排队的一种顺序，使得 $n$ 个人的平均等待时间最小。
+一个人的等待时间不包括他的接水时间。
+如果两个人接水的时间相同，编号更小的人应当排在前面。</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我试着比较两个相邻选择，但不知道要看总目标值还是局部贡献，感觉还没形成交换理由。样例能跟，可是一换顺序我就不知道为什么不会变差，也不知道该先固定哪个局部对象来比较。</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>学生：我觉得可以按某种规则先选一个局部最优，但不知道如果换一种选择顺序，会不会影响最终答案。 我不确定该看题面的哪个限制，所以后面越写越乱。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。
-AI：先别急着要完整做法。围绕《[NOISG 2024 Prelim] Part》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
+          <t>学生：我知道可能要让时间短的人先接水，但不会证明。交换两个人顺序时，到底该比较谁的等待时间变化？
+AI：先别急着要完整做法。围绕《排队接水》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
 学生：我感觉自己在套模板，不确定这个判断是不是对应题意。
 AI：那先别扩大范围。继续只看这一小步：你先比较两个相邻选择互换以后，目标值会不会变差。</t>
         </is>
@@ -10498,36 +10493,36 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我试着比较两个相邻选择，但不知道要看总目标值还是局部贡献，感觉还没形成交换理由。样例能跟，可是一换顺序我就不知道为什么不会变差，也不知道该先固定哪个局部对象来比较。</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>交换理由</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>缺少把局部选择与全局目标、不变量或交换论证连接起来的正确性桥。</t>
+          <t>缺少把两个相邻人的顺序交换与总等待时间变化连接起来的正确性桥。</t>
         </is>
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先比较两个局部选择的后果。
-回复引导学生寻找保持不变的量或可以交换的局部结构。
-回复不直接给完整证明。</t>
+          <t>回复让学生只比较相邻两个人 A、B 交换前后的等待时间贡献。
+回复引导学生找出哪个局部顺序不会让总等待时间变大。
+回复不直接给完整排序规则证明或完整贪心结论。</t>
         </is>
       </c>
       <c r="V38" s="2" t="inlineStr">
@@ -10588,55 +10583,61 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P10728</t>
+          <t>https://www.luogu.com.cn/problem/P1080</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>luogu_p10728_correctness_invariant</t>
+          <t>luogu_p1080_correctness_invariant</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOISG 2023 Qualification] Swords
-来源：洛谷 P10728
-题意摘录：YH 有 $n$ 把剑，第 $i$ 把剑的攻击力为 $a_i$，防御能力为 $b_i$。
-对于一把剑 $i$，如果存在一个 $j(j \not = i)$，使得 $a_i\le a_j$ 且 $b_i\le b_j$，那么 YH 就认为这把剑是无用的。反之，他就认为这把剑是有用的。
-在本题中，我们保证，不可能找到两把剑 $i,j$，使得 $a_i=a_j$ 且 $b_i=b_j$。
-请你帮助 YH 求出这 $n$ 把剑中，有用的剑的数量。
-输入格式摘录：第一行，一个整数 $n$。
-接下来 $n$ 行，每行两个整数 $a_i,b_i$，表示第 $i$ 把剑形的攻击力和防御能力。
-输出格式摘录：一个整数，表示有用的剑**的数量**。
-样例输入：3
-2 3
-1 3
-5 3
-样例输出：1
-数据范围/提示摘录：|$\text{Subtask}$|分值|特殊性质|
-|:-:|:-:|:-:|
-|$1$|$11$|$n\le500$|
-|$2$|$21$|$a_i,b_i\le500$|
-|$3$|$34$|$a_i=i$|
-|$4$|$25$|对于每一个 $1\le i&lt;j\le n$，有 $a_i\not =a_j$|
-|$5$|$9$|无|
-对于所有数据，$1\le n\le100000,1\le a_i,b_i\le10^9$。</t>
+          <t>题目：[NOIP 2012 提高组] 国王游戏
+来源：洛谷 P1080
+题意摘录：恰逢 H 国国庆，国王邀请 $n$ 位大臣来玩一个有奖游戏。首先，他让每个大臣在左、右手上面分别写下一个整数，国王自己也在左、右手上各写一个整数。然后，让这 $n$ 位大臣排成一排，国王站在队伍的最前面。排好队后，所有的大臣都会获得国王奖赏的若干金币，每位大臣获得的金币数分别是：排在该大臣前面的所有人的左手上的数的乘积除以他自己右手上的数，然后向下取整得到的结果。
+国王不希望某一个大臣获得特别多的奖赏，所以他想请你帮他重新安排一下队伍的顺序，使得获得奖赏最多的大臣，所获奖赏尽可能的少。注意，国王的位置始终在队伍的最前面。
+输入格式摘录：第一行包含一个整数 $n$，表示大臣的人数。
+第二行包含两个整数 $a$ 和 $b$，之间用一个空格隔开，分别表示国王左手和右手上的整数。
+接下来 $n$ 行，每行包含两个整数 $a$ 和 $b$，之间用一个空格隔开，分别表示每个大臣左手和右手上的整数。
+输出格式摘录：一个整数，表示重新排列后的队伍中获奖赏最多的大臣所获得的金币数。
+样例输入：3 
+1 1 
+2 3 
+7 4 
+4 6
+样例输出：2
+数据范围/提示摘录：**【输入输出样例说明】**
+按 $1$、$2$、$3$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $1$、$3$、$2$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $2$、$1$、$3$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；
+按 $2$、$3$、$1$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $9$；
+按 $3$、$1$、$2$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $2$；  
+按 $3$、$2$、$1$ 这样排列队伍，获得奖赏最多的大臣所获得金币数为 $9$。
+因此，奖赏最多的大臣最少获得 $2$ 个金币，答案输出 $2$。
+**【数据范围】**
+对于 $20\%$ 的数据，有 $1 \le n \le 10,0 &lt; a,b &lt; 8$；
+对于 $40\%$ 的数据，有 $1 \le n \le 20,0 &lt; a,b &lt; 8$；
+对于 $60\%$ 的数据，有 $1 \le n \le 100$；
+对于 $60\%$ 的数据，保证答案不超过 $10^9$；
+对于 $100\%$...</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P10728《[NOISG 2023 Qualification] Swords》：YH 有 $n$ 把剑，第 $i$ 把剑的攻击力为 $a_i$，防御能力为 $b_i$。
-对于一把剑 $i$，如果存在一个 $j(j \not = i)$，使得 $a_i\le a_j$ 且 $b_i\le b_j$，那么 YH 就认为这把剑是无用的。反之，他就认为这把剑是有用的。...</t>
+          <t>洛谷 P1080《[NOIP 2012 提高组] 国王游戏》：恰逢 H 国国庆，国王邀请 $n$ 位大臣来玩一个有奖游戏。首先，他让每个大臣在左、右手上面分别写下一个整数，国王自己也在左、右手上各写一个整数。然后，让这 $n$ 位大臣排成一排，国王站在队伍的最前面。排好队后，所有的大臣都会获得国王奖赏的若干金币，每位大臣获得的金币数分别是：排在该大臣前面的所有人的左手上的数的乘积除以他自己右手上的数，然后向下取整得到的结果。
+国王不希望某一个大臣获得特别多的奖赏，所以他想请你帮他重新安排一下队伍的顺序，使得获得奖赏最多的大臣，所获奖赏...</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>如果把这两个选择顺序换一下，我不确定哪个量不会变差。样例能跟，但证明这一步不会写，我想先确认比较的对象到底是哪一个，再判断全局目标有没有受影响。</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>学生：我能写出一个看起来合理的策略，但说不清它保持了什么不变量，所以不敢相信。 我看样例能跟上，但换成自己写就不知道该先确认哪一步。 我现在不知道该先看思路还是先看代码，所以越写越乱。
-AI：先别急着要完整做法。围绕《[NOISG 2023 Qualificatio》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
+          <t>学生：国王游戏里我能想到要排序，但不知道为什么这样排。只交换相邻两个大臣时，应该比较哪几个奖励值？
+AI：先别急着要完整做法。围绕《[NOIP 2012 提高组] 国王游戏》，我们只拆当前一小步：你先比较两个相邻选择互换以后，目标值会不会变差。
 学生：我能说出一点，但还是不知道它怎么落到这题里。
 AI：好，我们就停在这个局部。你先回答一个更小的问题：你先比较两个相邻选择互换以后，目标值会不会变差。</t>
         </is>
@@ -10653,36 +10654,36 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>如果把这两个选择顺序换一下，我不确定哪个量不会变差。样例能跟，但证明这一步不会写，我想先确认比较的对象到底是哪一个，再判断全局目标有没有受影响。</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不会变差</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>缺少把局部选择与全局目标、不变量或交换论证连接起来的正确性桥。</t>
+          <t>缺少把相邻两个大臣交换前后的局部最坏奖励与全局最大值控制连接起来的正确性桥。</t>
         </is>
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先比较两个局部选择的后果。
-回复引导学生寻找保持不变的量或可以交换的局部结构。
-回复不直接给完整证明。</t>
+          <t>回复让学生固定其他人，只比较相邻两个大臣交换前后的局部最坏奖励。
+回复引导学生观察交换只影响这两个位置相关的奖励项。
+回复不直接给完整排序关键字或完整交换证明。</t>
         </is>
       </c>
       <c r="V39" s="2" t="inlineStr">
@@ -10795,7 +10796,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 我对《[CSP-J 2024] 小木棍》的整体思路大概能跟，但代码里这个更新顺序一变结果就不一样。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我能猜到要保持某个不变量，但不知道相邻两步交换后到底保持了什么，为什么答案不会更差。现在我只是凭直觉说贪心可行，换一个样例就说不清理由，也不知道该比较哪两个局部方案。</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -10818,17 +10819,17 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 我对《[CSP-J 2024] 小木棍》的整体思路大概能跟，但代码里这个更新顺序一变结果就不一样。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>我能猜到要保持某个不变量，但不知道相邻两步交换后到底保持了什么，为什么答案不会更差。现在我只是凭直觉说贪心可行，换一个样例就说不清理由，也不知道该比较哪两个局部方案。</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不变量</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S40" s="2" t="inlineStr">
@@ -10838,9 +10839,9 @@
       </c>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U40" s="2" t="inlineStr">
@@ -10945,7 +10946,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我现在只会说这个贪心看起来对，但说不出局部选择换一下会不会影响全局目标。能不能先让我比较一个很小的相邻交换，看交换前后哪个量没有变差，再决定证明方向？</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -10968,17 +10969,17 @@
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道应该打印哪个中间量，别一上来就整段重写。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我现在只会说这个贪心看起来对，但说不出局部选择换一下会不会影响全局目标。能不能先让我比较一个很小的相邻交换，看交换前后哪个量没有变差，再决定证明方向？</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>全局目标</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S41" s="2" t="inlineStr">
@@ -10988,9 +10989,9 @@
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U41" s="2" t="inlineStr">
@@ -11108,7 +11109,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我想用交换法想这题，但卡在比较两种相邻选择：到底要证明哪个指标不变或不变差？我怕一上来就写证明会变成背模板，所以想先看一个局部比较，再慢慢推广到整体。</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -11131,17 +11132,17 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我改过一次循环范围，样例还是不稳，所以怀疑不是单纯少写一行。 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。</t>
+          <t>我想用交换法想这题，但卡在比较两种相邻选择：到底要证明哪个指标不变或不变差？我怕一上来就写证明会变成背模板，所以想先看一个局部比较，再慢慢推广到整体。</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>不变差</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S42" s="2" t="inlineStr">
@@ -11151,9 +11152,9 @@
       </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>no_full_proof
-no_complete_exchange_argument
-no_full_solution</t>
+          <t>Do not provide the full correctness proof
+Do not give the full exchange argument or greedy proof
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U42" s="2" t="inlineStr">
@@ -11315,9 +11316,9 @@
       </c>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr">
@@ -11469,9 +11470,9 @@
       </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
@@ -11613,9 +11614,9 @@
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_full_keypress_mapping_table</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not provide the full keypress mapping table</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -11750,7 +11751,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>立体图里一个方块画到字符图上时，我不知道单个字符位置到底对应题面里的哪一格、哪条边或哪个角。样例图我能看，但自己画时坐标就乱了，尤其不知道先核对哪个局部字符。</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -11773,36 +11774,36 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>我好像连一个字符该怎么处理都没懂，后面的循环就更接不上。 我现在看《[NOIP 2008 普及组] 立体图》时连字符、空格和计数范围都没对上，所以代码只能靠猜。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。</t>
+          <t>立体图里一个方块画到字符图上时，我不知道单个字符位置到底对应题面里的哪一格、哪条边或哪个角。样例图我能看，但自己画时坐标就乱了，尤其不知道先核对哪个局部字符。</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>没懂</t>
+          <t>单个字符位置</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t>缺少把题面范围、数组下标、初始可达状态和变量类型对应起来的实现边界桥。</t>
+          <t>缺少把输出图中单个字符位置、题面方块的格子/边/角以及循环坐标对应起来的实现边界桥。</t>
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>no_complete_code_patch
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not rewrite the full code for the student
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U46" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先用最小样例核对一个下标、初始值或类型范围。
-回复把注意力放在一个实现边界上。
-回复不直接给完整代码补丁。</t>
+          <t>回复先选一个最小方块或一个字符位置，让学生判断它对应题面中的哪一格、哪条边或哪个角。
+回复把注意力放在输出坐标、字符位置和题面对象的局部映射上。
+回复不直接给完整画图代码或完整字符模板。</t>
         </is>
       </c>
       <c r="V46" s="2" t="inlineStr">
@@ -11921,7 +11922,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>你说的维护量/不变量我没太理解，能不能先说它在题面里对应什么？ 我可能不是这一步不会写，而是前面那个概念就没有搭起来。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我知道要调试，但不知道“最小反例”该怎么选。能不能先让我挑一个很小输入，看哪个中间量应该是多少？我现在不是想改完整代码，只想把错误缩小到一步。</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -11944,17 +11945,17 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>你说的维护量/不变量我没太理解，能不能先说它在题面里对应什么？ 我可能不是这一步不会写，而是前面那个概念就没有搭起来。 我自己试着顺了一遍样例，但只能看到表面过程，看不出为什么下一步一定要这样接。</t>
+          <t>我知道要调试，但不知道“最小反例”该怎么选。能不能先让我挑一个很小输入，看哪个中间量应该是多少？我现在不是想改完整代码，只想把错误缩小到一步。</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>没太理解</t>
+          <t>最小反例</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S47" s="2" t="inlineStr">
@@ -11964,9 +11965,9 @@
       </c>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U47" s="2" t="inlineStr">
@@ -12074,7 +12075,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。 我现在愿意自己继续推，但需要一个不会直接暴露答案的提示。最好是让我对着一个最小样例说出下一步，而不是直接告诉我完整模板。</t>
+          <t>这题我样例能跟一点，但不知道该先手算哪一秒、哪个魔法值或距离变量。能先帮我把检查点缩小吗？我现在调试时只会整段跑，看到 WA 也不知道是闪烁、休息还是跑步那一步错了。最好先让我对一个很小时间点写出一个中间值，而不是直接告诉我完整做法。比如只看前两三秒，我也不确定该记录“当前最远距离”还是“剩余魔法”。</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -12097,17 +12098,17 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫可行性/状态语义？这个词我没太懂。 如果可以的话，能不能先用这题里的一个小对象解释这个词，而不是直接讲完整做法？ 我希望先确认这个小关系，因为一旦这里错了，后面写代码就会一直靠猜。 我现在愿意自己继续推，但需要一个不会直接暴露答案的提示。最好是让我对着一个最小样例说出下一步，而不是直接告诉我完整模板。</t>
+          <t>这题我样例能跟一点，但不知道该先手算哪一秒、哪个魔法值或距离变量。能先帮我把检查点缩小吗？我现在调试时只会整段跑，看到 WA 也不知道是闪烁、休息还是跑步那一步错了。最好先让我对一个很小时间点写出一个中间值，而不是直接告诉我完整做法。比如只看前两三秒，我也不确定该记录“当前最远距离”还是“剩余魔法”。</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>我有点懵，什么叫</t>
+          <t>检查点</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S48" s="2" t="inlineStr">
@@ -12117,9 +12118,9 @@
       </c>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U48" s="2" t="inlineStr">
@@ -12254,7 +12255,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[CSP-J 2021] 网络连接》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。 我已经试过按题面手算一个小例子，但算到中间就不知道该记录哪个量，代码里也不知道该检查哪一行。你先别直接给完整公式，帮我把这个小关系拆清楚就行。</t>
+          <t>网络连接这题我不知道该造哪种最小坏地址来查错，也不知道该先检查解析结果还是连接表。比如样例能过，但一遇到前导零、端口范围或重复 Server，我就不知道该打印哪一步。你先别直接改代码，帮我把一个最小坏样例和要看的中间结果定下来。最好只选一种错误类型，让我判断它应该先输出 ERR、FAIL 还是某个编号。</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -12277,17 +12278,17 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>我好像连这一格记录的“含义”都没懂，后面的公式就更接不上。 我现在看《[CSP-J 2021] 网络连接》时连这个基础关系都没对上，所以后面的转移/维护都接不上。 现在我最怕的是把一个模板套上去，结果换成别的数据就又不知道该怎么判断。 我已经试过按题面手算一个小例子，但算到中间就不知道该记录哪个量，代码里也不知道该检查哪一行。你先别直接给完整公式，帮我把这个小关系拆清楚就行。</t>
+          <t>网络连接这题我不知道该造哪种最小坏地址来查错，也不知道该先检查解析结果还是连接表。比如样例能过，但一遇到前导零、端口范围或重复 Server，我就不知道该打印哪一步。你先别直接改代码，帮我把一个最小坏样例和要看的中间结果定下来。最好只选一种错误类型，让我判断它应该先输出 ERR、FAIL 还是某个编号。</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>没懂</t>
+          <t>最小坏地址</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>学生暴露前置概念断层，需要先补基础概念。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S49" s="2" t="inlineStr">
@@ -12297,9 +12298,9 @@
       </c>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t>no_direct_bug_fix
-no_complete_code_patch
-no_full_solution</t>
+          <t>Do not directly identify and fully fix the bug
+Do not rewrite the full code for the student
+Do not provide the full solution</t>
         </is>
       </c>
       <c r="U49" s="2" t="inlineStr">
@@ -12453,9 +12454,9 @@
       </c>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U50" s="2" t="inlineStr">
@@ -12603,9 +12604,9 @@
       </c>
       <c r="T51" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U51" s="2" t="inlineStr">
@@ -12779,9 +12780,9 @@
       </c>
       <c r="T52" s="2" t="inlineStr">
         <is>
-          <t>no_full_solution
-no_full_code
-no_direct_answer_confirmation</t>
+          <t>Do not provide the full solution
+Do not provide full code
+Do not directly confirm the full answer, algorithm, or solution path</t>
         </is>
       </c>
       <c r="U52" s="2" t="inlineStr">
@@ -13355,9 +13356,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -13478,9 +13479,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -13611,9 +13612,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -13736,9 +13737,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -13865,9 +13866,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -14000,9 +14001,9 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>no_exact_state_definition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact full state/variable definition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
@@ -14581,9 +14582,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -14713,9 +14714,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -14839,9 +14840,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -14981,9 +14982,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -15155,9 +15156,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_exact_recurrence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not write the full recurrence or transition equation
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -15752,9 +15753,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -15896,9 +15897,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -16036,9 +16037,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -16196,9 +16197,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -16338,9 +16339,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_complete_check_condition
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete check/predicate condition
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -16935,9 +16936,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -17082,9 +17083,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -17236,9 +17237,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -17391,9 +17392,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -17537,9 +17538,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_exact_boundary_update_rule
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the exact boundary update or loop-order rule
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -18178,9 +18179,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -18329,9 +18330,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -18483,9 +18484,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -18635,9 +18636,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -18779,9 +18780,9 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_complete_model_mapping
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full modeling mapping
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -19367,7 +19368,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>对 [L,R] 加 X 的影响我能看出来，但不知道标记应该落在 L、R 还是抵消位置。这里我经常写成凭感觉加减。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -19388,17 +19389,17 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>对 [L,R] 加 X 的影响我能看出来，但不知道标记应该落在 L、R 还是抵消位置。这里我经常写成凭感觉加减。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>另一边</t>
+          <t>抵消位置</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -19408,9 +19409,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -19540,7 +19541,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我能看出一次操作会影响一路上的值，但不知道哪些位置是直接加，哪些位置是为了抵消。这里换一个询问我就乱。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -19561,17 +19562,17 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我能看出一次操作会影响一路上的值，但不知道哪些位置是直接加，哪些位置是为了抵消。这里换一个询问我就乱。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>为了抵消</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -19581,9 +19582,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -19703,7 +19704,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>单个星球或区间的影响我能跟，但要把很多次影响汇总起来时，我不知道应该在哪些位置打标记。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -19724,17 +19725,17 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>单个星球或区间的影响我能跟，但要把很多次影响汇总起来时，我不知道应该在哪些位置打标记。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>打标记</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -19744,9 +19745,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -19859,7 +19860,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>路径上的贡献怎么累起来我懂一点，但到前缀汇总或公共点附近时，不知道加减点应该放在哪里。</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -19880,17 +19881,17 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>是不是只要当前判断成立，就往另一边继续找？我有点乱。 我现在更像在猜模板。</t>
+          <t>路径上的贡献怎么累起来我懂一点，但到前缀汇总或公共点附近时，不知道加减点应该放在哪里。</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>另一边</t>
+          <t>加减点</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -19900,9 +19901,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_complete_marking_formula
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the complete marking/contribution formula
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -20457,7 +20458,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我知道要 update/query，但不知道结构里每个节点到底该存什么摘要，才能回答题目要的数量或最值。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -20478,17 +20479,17 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>应该是反过来吧？如果 true 就说明这一边不用管了？ 我感觉方向反了。</t>
+          <t>我知道要 update/query，但不知道结构里每个节点到底该存什么摘要，才能回答题目要的数量或最值。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>存什么摘要</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -20498,9 +20499,9 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -20619,7 +20620,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>一次修改之后，节点里的值要怎么保持正确我没想清。查询时为什么能直接拿这些维护量拼出答案？</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -20640,17 +20641,17 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>我是不是该把满足的那一边排除掉？感觉有点反。 边界一换我就乱了。</t>
+          <t>一次修改之后，节点里的值要怎么保持正确我没想清。查询时为什么能直接拿这些维护量拼出答案？</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>反</t>
+          <t>维护量</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>学生给出方向性判断，但明显不稳定。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -20660,9 +20661,9 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -20775,7 +20776,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道该打印哪个量。</t>
+          <t>我写了个小版本，query 输出和手算差一点。我想先知道一次 update 后，结构里哪个摘要量应该发生变化。</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -20796,17 +20797,17 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我写了个小版本，输出和手算差一点，不知道该先查哪一个中间量。 我想先知道该打印哪个量。</t>
+          <t>我写了个小版本，query 输出和手算差一点。我想先知道一次 update 后，结构里哪个摘要量应该发生变化。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>中间量</t>
+          <t>摘要量</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -20816,9 +20817,9 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -20943,7 +20944,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我怀疑不是单纯少写一行。</t>
+          <t>我不太明白查询为什么能由这些维护量拼出来。是不是要先确认每个节点维护的对象和合并含义？</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -20964,17 +20965,17 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我按这个想法写了一点，但样例第二个过不去，感觉边界或者更新顺序有问题。 我怀疑不是单纯少写一行。</t>
+          <t>我不太明白查询为什么能由这些维护量拼出来。是不是要先确认每个节点维护的对象和合并含义？</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>合并含义</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -20984,9 +20985,9 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -21054,97 +21055,106 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.luogu.com.cn/problem/P2672</t>
+          <t>https://www.luogu.com.cn/problem/P3374</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>luogu_p2672_data_structure_operation_semantics</t>
+          <t>luogu_p3374_data_structure_operation_semantics</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>题目：[NOIP 2015 普及组] 推销员
-来源：洛谷 P2672
-题意摘录：阿明是一名推销员，他奉命到螺丝街推销他们公司的产品。螺丝街是一条死胡同，出口与入口是同一个，街道的一侧是围墙，另一侧是住户。螺丝街一共有 $N$ 家住户，第 $i$ 家住户到入口的距离为 $S_i$ 米。由于同一栋房子里可以有多家住户，所以可能有多家住户与入口的距离相等。阿明会从入口进入，依次向螺丝街的 $X$ 家住户推销产品，然后再原路走出去。
-阿明每走 $1$ 米就会积累 $1$ 点疲劳值，向第 $i$ 家住户推销产品会积累 $A_i$ 点疲劳值。阿明是工作狂，他想知道，对于不同的 $X$，在不走多余的路的前提下，他最多可以积累多少点疲劳值。
-输入格式摘录：第一行有一个正整数 $N$，表示螺丝街住户的数量。
-接下来的一行有 $N$ 个非负整数，其中第 $i$ 个整数 $S_i$ 表示第 $i$ 家住户到入口的距离。数据保证 $S_1 \le S_2 \le \cdots \le S_n &lt;10^8$。
-接下来的一行有 $N$ 个正整数，其中第 $i$ 个整数 $A_i$ 表示向第 $i$ 户住户推销产品会积累的疲劳值。数据保证 $A_i&lt;1000$。
-输出格式摘录：输出 $N$ 行，每行一个正整数，第 $i$ 行整数表示当 $X=i$ 时，阿明最多积累的疲劳值。
-样例输入：5
-1 2 3 4 5
-1 2 3 4 5
-样例输出：15
-19
-22
-24
-25
-数据范围/提示摘录：**输入输出样例 1 说明**
-$X=1$：向住户 $5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值为 $5$，总疲劳值为 $15$。
-$X=2$：向住户 $4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值为 $4+5$，总疲劳值为 $5+5+4+5=19$。
-$X=3$：向住户 $3,4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值 $3+4+5$，总疲劳值为 $5+5+3+4+5=22$。
-$X=4$：向住户 $2,3,4,5$ 推销，往返走路的疲劳值为 $5+5$，推销的疲劳值 $2+3+4+5$，总疲劳值 $5+5+2+3+4+5=24$。...</t>
+          <t>题目：【模板】树状数组 1
+来源：洛谷 P3374
+题意摘录：如题，已知一个数列，你需要进行下面两种操作：
+- 将某一个数加上 $x$；
+- 求出某区间每一个数的和。
+输入格式摘录：第一行包含两个正整数 $n,m$，分别表示该数列数字的个数和操作的总个数。   
+第二行包含 $n$ 个用空格分隔的整数，其中第 $i$ 个数字表示数列第 $i$ 项的初始值。
+接下来 $m$ 行每行包含 $3$ 个整数，表示一个操作，具体如下：
+- `1 x k`  含义：将第 $x$ 个数加上 $k$；
+- `2 x y`  含义：输出区间 $[x,y]$ 内每个数的和。
+输出格式摘录：输出包含若干行整数，即为所有操作 $2$ 的结果。
+样例输入：5 5
+1 5 4 2 3
+1 1 3
+2 2 5
+1 3 -1
+1 4 2
+2 1 4
+样例输出：14
+16
+数据范围/提示摘录：【数据范围】
+对于 $30\%$ 的数据，$1 \le n \le 8$，$1\le m \le 10$；   
+对于 $70\%$ 的数据，$1\le n,m \le 10^4$；   
+对于 $100\%$ 的数据，$1\le n,m \le 5\times 10^5$，$1\le x\le y\le n$，$-2^{31}\le k&lt;2^{31}$。
+数据保证对于任意时刻，$a$ 的任意子区间（包括长度为 $1$ 和 $n$ 的子区间）和均在 $[-2^{31}, 2^{31})$ 范围内。
+样例说明：
+ ![](https://cdn.luogu.com.cn/upload/pic/2256.png) 
+故输出结果 $14$ 和 $16$。</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>洛谷 P2672《[NOIP 2015 普及组] 推销员》：阿明是一名推销员，他奉命到螺丝街推销他们公司的产品。螺丝街是一条死胡同，出口与入口是同一个，街道的一侧是围墙，另一侧是住户。螺丝街一共有 $N$ 家住户，第 $i$ 家住户到入口的距离为 $S_i$ 米。由于同一栋房子里可以有多家住户，所以可能有多家住户与入口的距离相等。...</t>
+          <t>洛谷 P3374《【模板】树状数组 1》：如题，已知一个数列，你需要进行下面两种操作：
+- 将某一个数加上 $x$；
+- 求出某区间每一个数的和。</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 更新顺序一变结果就不同。</t>
+          <t>更新后结果不稳，我怀疑不是下标问题，而是某个维护量没更新对。应该先检查哪个摘要量？</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>学生：我不清楚一次修改以后，结构里哪些量需要跟着变。 我总觉得差一步。
-AI：先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>学生：我知道有单点加和区间求和，但树状数组里面维护的到底是什么？update 之后 query 为什么还能算区间和？
+AI：先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>先别急着要完整做法。围绕《[NOIP 2015 普及组] 推销员》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
+          <t>先别急着要完整做法。围绕《【模板】树状数组 1》，我们只拆当前一小步：你先说一次 update/query 之后，结构里应该保持什么摘要信息。</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>我把这一步写进代码了，不过有一组样例不对，可能是初始化或者下标错了。 更新顺序一变结果就不同。</t>
+          <t>更新后结果不稳，我怀疑不是下标问题，而是某个维护量没更新对。应该先检查哪个摘要量？</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>样例</t>
+          <t>维护量</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>学生有尝试和错误证据，但还没有定位到最小桥。</t>
+          <t>Coach A round1 case/source review: revised current student reply to align with the bridge bucket and prior scaffold.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>缺少把数据结构节点、集合或队列中的值与题目需要查询/更新的信息对应起来的关系。</t>
+          <t>缺少把单点修改、前缀和查询以及数据结构内部维护的摘要量对应起来的关系。</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>no_complete_operation_sequence
-no_full_solution
-no_direct_current_bridge</t>
+          <t>Do not give the full operation sequence or data-structure workflow
+Do not provide the full solution
+Do not directly complete the student's current missing bridge</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>回复让学生先说明一次 update/query 后应保持什么摘要不变量。
-回复用一个极小局部操作检查维护语义。
-回复不直接给完整数据结构操作模板。</t>
+          <t>回复让学生先说明一次 update 后哪些前缀/摘要信息应随之改变。
+回复用一个极小数组检查 query 需要从哪些维护量组合出区间和。
+回复不直接给完整树状数组模板或完整 lowbit 操作序列。</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">

</xml_diff>